<commit_message>
cron VPS + lessons L26/L27 + alpha guard confirm
Cron VPS 5.223.67.21: collect_spot_daily 01:05, collect_alpha_spot 01:10
(sau export 00:50). Tape HOÃN (B3: one-shot REST không cover full-day).
paths.py: thêm spot_klines_partition_path + spot_tape_partition_path.
LESSONS L-26 (file canonical), L-27 (fn=1 mapping guard) — GHI NHẬN.
CLAUDE.md: 3 dòng kỷ luật skip-permissions + Nansen env lock.
Alpha guard B4 PASS — code đã đủ guard + comment.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/case_files/CASE_INDEX.xlsx
+++ b/docs/case_files/CASE_INDEX.xlsx
@@ -1,19 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="INDEX" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LESSONS" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MM_BOOK" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PHAN_VAI" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="INDEX" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="LESSONS" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="MM_BOOK" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="PHAN_VAI" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -40,7 +39,7 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
       <sz val="10"/>
     </font>
     <font>
@@ -62,22 +61,22 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00404040"/>
+        <fgColor rgb="FF404040"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E2EFDA"/>
+        <fgColor rgb="FFE2EFDA"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FCE4EC"/>
+        <fgColor rgb="FFFCE4EC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F2F2F2"/>
+        <fgColor rgb="FFF2F2F2"/>
       </patternFill>
     </fill>
   </fills>
@@ -91,17 +90,18 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="FFBFBFBF"/>
       </left>
       <right style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="FFBFBFBF"/>
       </right>
       <top style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="FFBFBFBF"/>
       </top>
       <bottom style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="FFBFBFBF"/>
       </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
@@ -131,7 +131,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -495,7 +495,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:K11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
@@ -504,13 +504,12 @@
     <col width="24" customWidth="1" min="5" max="5"/>
     <col width="11" customWidth="1" min="6" max="6"/>
     <col width="24" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="8" max="9"/>
     <col width="16" customWidth="1" min="10" max="10"/>
     <col width="42" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="16.8" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>FRESHWATCH CASE INDEX — hub tong: danh sach case + LESSONS + MM_BOOK + PHAN_VAI</t>
@@ -991,19 +990,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:H31"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="70" customWidth="1" min="4" max="4"/>
+    <col width="169.5546875" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="34" customWidth="1" min="6" max="6"/>
-    <col width="42" customWidth="1" min="7" max="7"/>
+    <col width="78.21875" bestFit="1" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="16.8" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>LESSONS LEARNED — hub bai hoc cross-case (append-only, khong xoa bai hoc cu)</t>
@@ -1053,6 +1052,11 @@
           <t>hanh_dong_tiep</t>
         </is>
       </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>MM</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="15" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
@@ -1532,6 +1536,524 @@
       <c r="G17" s="4" t="inlineStr">
         <is>
           <t>them cot case_id vao Zone B (viec tay 1 phut)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>L-14</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>ESPORTS + twelve_cases_ref</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Wash-by-crash: crowd flush khi gia sap (long dung lo, short mo them) -&gt; gLSR tang -&gt; squeeze nguoc gia bat, short ket = nhien lieu pump. Signal: gia sap + gLSR TANG dong thoi = tiem nang squeeze nguoc (nguoc chieu voi wash-by-rally L-11)</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>thesis</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>GHI NHAN</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>kiem xac nhan wash-by-crash tren ESPORTS daily log khi backfill</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>L-15</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>twelve_cases_ref + BANK/TAG</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Bait-probe: MM tao probe nho (vol spike ngan + gia retreat) do phan ung crowd. Crowd khong khang cu = san sang markup; crowd short ngay = can them wash. Probe khac markup that: khong co vol sustained sau probe</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>thesis</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>GHI NHAN</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>tag probe events trong EVENTS log (BANK/TAG neu thay pattern)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>L-16</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>twelve_cases_ref + BR/EVAA</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>M2 dao dau (div_raw tu &gt;1 xuong &lt;1 = acc_r vuot pos_r): smart money khong con long bias hon crowd, crowd bat dau hold nhieu hon. Dao dau M2 = phase distribution bat dau. BR: div_raw 1.114-&gt;0.51 qua 10 ngay; EVAA tuong tu</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>dinh luat</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>GHI NHAN</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>flag M2-flip trong DAILY log; xet lam trigger STAND_ASIDE review</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>L-17</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>ESPORTS + twelve_cases_ref</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Squeeze chet khi nhien lieu chet: gLSR quay dau (gLSR_slope_5d doi dau) = short positions dong/chuyen long, het nhien lieu pump. Theo doi glsr_slope_5d: duong-&gt;am = tank can; squeeze khong the keo dai sau khi crowded-short tan</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>dinh luat</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>GHI NHAN</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>them glsr_slope_5d vao S1 handover checklist</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>L-18</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>u50_verdicts §2</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>u50 §2 — Fire khong = markup ngay: can dong thoi (1) MM phase gom/markup (khong phai phan phoi), (2) crowd structure sach (gLSR hop ly), (3) OI khong PEAK. Thieu 1/3 = low-conviction, khong arm. Fire-without-phase-check dung ~40% tu 50-verdict review</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>thesis</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>GHI NHAN</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>them phase_check vao ARM checklist truoc khi ARM</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>L-19</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>u50_verdicts §3</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>u50 §3 — He thong thieu phase-context filter: signal fire ban giong nhau o phase gom va phan phoi. Can phase_tag (ACCUMULATE/MARKUP/DISTRIBUTE) tu oi_cycle_pos + div_raw de loc false-fire trong phan phoi. ~30% fire trong DISTRIBUTE la false theo u50</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>process</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>GHI NHAN</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>thiet ke phase_tag inference (oi_cycle_pos + div_raw + M2) — no P2</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>L-20</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>u50_verdicts §6 + TAG/BR 29/07</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>u50 §6 tu-ha-cap: agent ha cap confidence + ghi low_conf=True khi: fn=1, data_bad=1, missing &gt;3 ngay trong window, hoac so chot tu 1 nguon khong kiem chung duoc. So bi ha cap khong duoc lam threshold ARM/FIRE</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>process</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>DA VAO CLAUDE.md (fn=1 rule)</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>mo rong tu-ha-cap cho data_bad flag (ngoai fn=1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>L-21</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>BR (an 30/07)</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>OI daily canonical = export Binance openInterestHist 00:00 UTC. So intraday (Coinglass/GMGN) chi vao EVENTS kem timestamp, khong vao DAILY. An 30/07: BR 4,634,000 (intraday) vs 3,782,263 (export 00:00) chenh 22%. Rule: mot cot DAILY mot so canonical</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>rule</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>DA VAO CLAUDE.md</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>khi co so OI: xac nhan nguon + gio chup truoc khi ghi DAILY</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>L-22</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>TAG+BR 28-29/07</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>fn=1 (native_1d low_conf) khong dung lam so chot ARM/FIRE. Fallback: Zone A aggregate tu ledger_v2.xlsx CAMPAIGNS, ghi ro Zone-A-agg. TAG 29/07: gLSR 1.81 (fn=1 SUSPECT) vs 1.61 (Zone-A-agg) — chenh 0.2 du dao nhan dinh toc do nap crowd</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>rule</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>DA VAO CLAUDE.md</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>khi fn&lt;6: tu dong dung Zone-A-agg + flag SUSPECT trong handover</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>L-23</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>TAG</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Fire margin mong -&gt; fade la kich ban xac suat cao: TAG 28/07 fire bien mong, ret_3d=-9.87%, crowd nap long vao duong gia xuong (gLSR 1.28-&gt;1.81). Invalidate som: gia khong confirm T+1/T+2 + gLSR tang tiep = WATCH-ha-nhiet, khong ARM lai som</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>thesis</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>GHI NHAN</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>them T+1/T+2 price-confirm check vao S1 handover (48h khong confirm = WATCH-ha-nhiet)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>L-24</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>BR/TAG (an 30/07)</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>oi_vs_med14 Excel != oi_vs_med14 signals.py (window ket thuc ngay khac). Moi so DAILY phai mang nhan: nguon + window cu the. Khong dung Excel calc lam proxy signals.py canonical. Hai nguoi doc hai so khac nhau cung ten = an tranh luan vo ich</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>rule</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>DA VAO CLAUDE.md (facts da chot)</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>moi oi_vs_med14 phai kem (signals.py, window=...) hoac (Excel, col X)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>L-25</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>BR+TAG (tai pham 30/07)</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Mot-nha-mot-data tai pham x2 trong session 30/07: (1) OI DAILY 2 so tu 2 nguon; (2) gLSR/div dung fn=1 raw thay vi aggregate canonical. Rule: moi cot DAILY mot nguon canonical khai bao tuong minh. &gt;=2 so cung metric -&gt; chon canonical + ghi an vao EVENTS</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>rule</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>DA VAO CLAUDE.md (KY LUAT)</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>audit cot DAILY hien tai: co cot nao 2 nguon khong khai bao khong?</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>L-26</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>BANK</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Backfill save nhầm file (_NEW suffix) do file gốc bị lock trong Excel — INDEX vẫn trỏ tên cũ → case_daily ghi vào file cũ (4 dòng) thay vì canonical (35 dòng). Fix: sau bất kỳ backfill nào, verify INDEX trỏ đúng canonical; canonical phải có đúng tên gốc.</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>process/rule</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>GHI NHAN</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>thêm bước verify file name + row count vào checklist sau backfill</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>L-27</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>BANK</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>fn=1 fallback (Zone-A-agg) chỉ dành cho cột taker_buy_pct — KHÔNG mượn sang gLSR/pos_r/acc_r. Metric ratio phải đến từ export CSV hoặc để TRỐNG + comment, không ghép chéo metric. Guard bằng assert EXPORT_COL_MAP tại import time trong case_daily.py.</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>rule</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>GHI NHAN</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>assert đã vào case_daily.py dòng sau FORMULA_COLS</t>
         </is>
       </c>
     </row>
@@ -1547,7 +2069,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E8"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="58" customWidth="1" min="2" max="2"/>
@@ -1556,7 +2078,7 @@
     <col width="50" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="16.8" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>SO MM CHUNG — van tay hanh vi cross-case (chuyen tu case_tracker.md §4 ve day)</t>
@@ -1717,14 +2239,13 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="55" customWidth="1" min="2" max="2"/>
-    <col width="55" customWidth="1" min="3" max="3"/>
+    <col width="55" customWidth="1" min="2" max="3"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="16.8" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>PHAN VAI LEDGER vs CASE TRACKER — duyet 30/07</t>
@@ -1739,7 +2260,7 @@
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="7" t="inlineStr"/>
+      <c r="A4" s="7" t="n"/>
       <c r="B4" s="8" t="inlineStr">
         <is>
           <t>LEDGER v2 (so cai NGANG)</t>

</xml_diff>

<commit_message>
lessons: sync rev.2 + renumber + L-34
- L-26/L-27 (agent session 30/07) → renumber L-32/L-33
- L-14..L-20: sua noi dung theo rev.2 (xoa so bia, doi ten L-16, them co che L-14/L-15)
- Chen L-26..L-31 moi: wrong-side fuel, M2 dao dau, tu-ha-cap narrative,
  alpha_vol_suspect, Bitget lech ngay, consolidation nguon
- Them L-34: PermissionError RAISE (cam silent-save ten khac)
- Ket qua: 34 bai, L-01..L-34 day du, khong trung ID
- Regenerate docs/lessons_learned.md (141 dong)
- Luu nguon: docs/lessons_rev2_source.md (operator approved)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/case_files/CASE_INDEX.xlsx
+++ b/docs/case_files/CASE_INDEX.xlsx
@@ -990,7 +990,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H31"/>
+  <dimension ref="A1:H38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1552,12 +1552,12 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>ESPORTS + twelve_cases_ref</t>
+          <t>TAG 08-09/07 + AKE 08-10/07</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Wash-by-crash: crowd flush khi gia sap (long dung lo, short mo them) -&gt; gLSR tang -&gt; squeeze nguoc gia bat, short ket = nhien lieu pump. Signal: gia sap + gLSR TANG dong thoi = tiem nang squeeze nguoc (nguoc chieu voi wash-by-rally L-11)</t>
+          <t>Dump manh + gLSR SAP &gt;=30%/&lt;=3d = wash-by-crash: mot phat an hai: don chi phi long + nap nhien lieu short (crowd short moi = nhien lieu re cho squeeze). La bien the crowd_flush thu nhat, doi xung L-11 (rally) va L-15 (bait). Phan biet ro voi L-26: gLSR SAP khi gia sap (wash) vs gLSR TANG khi gia sap (wrong-side fuel)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1567,12 +1567,12 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>GHI NHAN</t>
+          <t>DA VAO yaml (crowd_flush cause=crash)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>kiem xac nhan wash-by-crash tren ESPORTS daily log khi backfill</t>
+          <t>phan biet ro voi L-26 (gLSR TANG khi gia sap = hien tuong nguoc, KHONG phai wash)</t>
         </is>
       </c>
     </row>
@@ -1589,12 +1589,12 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>twelve_cases_ref + BANK/TAG</t>
+          <t>BANK 02/07 + BASED 01&amp;09/07 + POWER 08-09/07</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Bait-probe: MM tao probe nho (vol spike ngan + gia retreat) do phan ung crowd. Crowd khong khang cu = san sang markup; crowd short ngay = can them wash. Probe khac markup that: khong co vol sustained sau probe</t>
+          <t>Vol spike &gt;=8x med14 + gia bi tu choi &lt;=2d = bait-probe: muc dich khong phai markup het ma la DAY crowd short nap nhien lieu squeeze. Sau bait canh gLSR sap trong &lt;=3d lam xac nhan; vol persistence T+1 phan biet bait vs ignition that</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1604,12 +1604,12 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>GHI NHAN</t>
+          <t>DA VAO yaml (crowd_flush cause=bait)</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>tag probe events trong EVENTS log (BANK/TAG neu thay pattern)</t>
+          <t>tag probe events trong EVENTS log khi thay pattern</t>
         </is>
       </c>
     </row>
@@ -1626,17 +1626,17 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>twelve_cases_ref + BR/EVAA</t>
+          <t>BR + EVAA + CLO</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>M2 dao dau (div_raw tu &gt;1 xuong &lt;1 = acc_r vuot pos_r): smart money khong con long bias hon crowd, crowd bat dau hold nhieu hon. Dao dau M2 = phase distribution bat dau. BR: div_raw 1.114-&gt;0.51 qua 10 ngay; EVAA tuong tu</t>
+          <t>div_raw truot tu &gt;1 xuong &lt;1 = vi the lon thu hep/dao long bias = chom phan phoi; flag STAND_ASIDE review; khong ARM sau div-flip neu chua co bang chung re-gom. LUU Y THUAT NGU: day KHONG phai 'M2 dao dau' — M2 la module CEX balance flow (xem L-27)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>dinh luat</t>
+          <t>thesis</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1646,7 +1646,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>flag M2-flip trong DAILY log; xet lam trigger STAND_ASIDE review</t>
+          <t>flag div-flip trong DAILY log; ho hang gan voi lsr_dist (da la suppressor yaml)</t>
         </is>
       </c>
     </row>
@@ -1663,12 +1663,12 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>ESPORTS + twelve_cases_ref</t>
+          <t>AKE + ESPORTS</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Squeeze chet khi nhien lieu chet: gLSR quay dau (gLSR_slope_5d doi dau) = short positions dong/chuyen long, het nhien lieu pump. Theo doi glsr_slope_5d: duong-&gt;am = tank can; squeeze khong the keo dai sau khi crowded-short tan</t>
+          <t>Squeeze/markup chet khi nhien lieu chet — hai cua dong an: (a) gLSR hoi ve ~1 (crowd short dau hang), (b) muc tieu cu the goc (TARGETED_SQUEEZE). Dang giu vi the ma mot trong hai bat = EXIT_NOW. [De xuat CHUA CALIB: thao tac hoa bang glsr_slope_5d doi dau — chua test case nao, glsr_slope_5d hien chi la cot hien thi (A5), khong phai gate]</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1678,12 +1678,12 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>GHI NHAN</t>
+          <t>DA VAO master plan §1 #5 + EXIT_NOW conditions</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>them glsr_slope_5d vao S1 handover checklist</t>
+          <t>neu muon slope-flip thanh trigger di duong proposal + calib nhu #17</t>
         </is>
       </c>
     </row>
@@ -1700,12 +1700,12 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>u50_verdicts §2</t>
+          <t>u50_verdicts §2 (n=18)</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>u50 §2 — Fire khong = markup ngay: can dong thoi (1) MM phase gom/markup (khong phai phan phoi), (2) crowd structure sach (gLSR hop ly), (3) OI khong PEAK. Thieu 1/3 = low-conviction, khong arm. Fire-without-phase-check dung ~40% tu 50-verdict review</t>
+          <t>Truoc ARM phai check du 3: (1) pha chu ky (nhin du px7/px14 + oi_cycle_pos, khong chi cua so 28d), (2) crowd structure (gLSR + dao ham — co tinh gan vo dung), (3) OI khong tai PEAK. Thieu 1/3 = low-conviction. KHONG trich dan % precision khi chua do — precedent dem that (n=...), cam noi %</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1720,7 +1720,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>them phase_check vao ARM checklist truoc khi ARM</t>
+          <t>phase_check vao ARM checklist; precision that do bang shadow-mode P2 + alerts_log</t>
         </is>
       </c>
     </row>
@@ -1737,12 +1737,12 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>u50_verdicts §3</t>
+          <t>u50 §2 + CLO/BLUAI/STAR (n=18)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>u50 §3 — He thong thieu phase-context filter: signal fire ban giong nhau o phase gom va phan phoi. Can phase_tag (ACCUMULATE/MARKUP/DISTRIBUTE) tu oi_cycle_pos + div_raw de loc false-fire trong phan phoi. ~30% fire trong DISTRIBUTE la false theo u50</t>
+          <t>Signal fire ban giong nhau o pha gom va pha phan phoi — can phase_tag (ACCUMULATE/MARKUP/DISTRIBUTE/UNKNOWN) tu oi_cycle_pos + div trend + glsr_slope de loc; den khi co phase_tag: moi fire phai kem phase check tay (L-18). Khong trich % false-rate khi chua do</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1752,12 +1752,12 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>GHI NHAN</t>
+          <t>GHI NHAN — no P2</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>thiet ke phase_tag inference (oi_cycle_pos + div_raw + M2) — no P2</t>
+          <t>thiet ke phase_tag inference trong P2</t>
         </is>
       </c>
     </row>
@@ -1774,12 +1774,12 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>u50_verdicts §6 + TAG/BR 29/07</t>
+          <t>TAG/BR 28-29/07</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>u50 §6 tu-ha-cap: agent ha cap confidence + ghi low_conf=True khi: fn=1, data_bad=1, missing &gt;3 ngay trong window, hoac so chot tu 1 nguon khong kiem chung duoc. So bi ha cap khong duoc lam threshold ARM/FIRE</t>
+          <t>fn=1 / data_bad=1 / missing &gt;3 ngay trong window / so tu 1 nguon khong kiem chung → low_conf=True; so bi ha cap KHONG lam threshold ARM/FIRE</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1996,17 +1996,17 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>BANK</t>
+          <t>ESPORTS hau-climax + TAG 29/07 + BLUAI</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Backfill save nhầm file (_NEW suffix) do file gốc bị lock trong Excel — INDEX vẫn trỏ tên cũ → case_daily ghi vào file cũ (4 dòng) thay vì canonical (35 dòng). Fix: sau bất kỳ backfill nào, verify INDEX trỏ đúng canonical; canonical phải có đúng tên gốc.</t>
+          <t>Gia sap/roi + gLSR TANG = crowd long bat dao = nhien lieu SAI phia — NGUOC han wash-by-crash (L-14: gLSR SAP). He qua: (a) leg-len ke tiep can lua long nay bi rua truoc, (b) con dang SUPPRESSED co pattern nay thi REMAIN, (c) khong doc nham thanh 'co nguoi gom'</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>process/rule</t>
+          <t>thesis</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -2016,7 +2016,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>thêm bước verify file name + row count vào checklist sau backfill</t>
+          <t>dieu kien tien quyet 'crowd flush truoc leg' ghi vao chot canh cac case dinh (TAG, BR, ESPORTS)</t>
         </is>
       </c>
     </row>
@@ -2033,27 +2033,286 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
+          <t>BTW vs BAS/TAG | AKE/IDOL</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>M2 (CEX balance flow) tu no KHONG mang y dinh — dau cua no do boi canh quyet: vi tri chu ky + funding regime + hanh vi gia. Chay M2 don le la An tron bay BTW. Suppressor o bat ky lop nao phu quyet moi bullish cua ca ba lop</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>dinh luat</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>DA VAO master plan §1 #1 + A1 (R4)</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>giu ten 'M2' doc quyen cho balance flow — khong dung cho div/ratio (an L-16 rev.1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>L-28</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>u50 §6 (AGT / HUMA-AT sync / listing 04-14)</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Moi narrative dung tren mot nguon phai kiem nguon goc (aggregator != klines; mep cua so = artifact ung vien). Narrative khong con dung duoc → RUT cong khai va GHI SO muc 'da tu ha cap' — de khong tu lua va khong tai sinh. Cu luan diem chi giu phan con dung tren bang chung</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>process</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>GHI NHAN — u50 §6 la mau chuan</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>moi report lon co muc 'bang chung da tu ha cap' nhu u50</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>L-29</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>OPN + HYPER (u50 §3a, n=2)</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>alpha_vol_suspect = vol_spot/vol_perp &gt; 3x → moi metric VOL SPOT cua con do ABSTAIN (khong wash-check, khong #17, khong bang chung dong tien); van dung depth/price/taker. takerBUY spot lech cuc doan (&lt;35% hoac &gt;70%) tren vol khong lo = hinh dang farming. Guard chi ha long tin, khong sinh bullish → ap ngay</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>guard</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>DA VAO amendment A6 (guard)</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>cot alpha_vol_suspect vao triage/snapshot khi build spot collector (P1.5)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>L-30</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>BLUAI + ARX (u50)</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Token venue_top=bitget: cam so sanh spot-vs-perp cung-ngay cho den khi bug lech ngay duoc xac minh/va; phan tich cross-market phai shift-test truoc. Ghi chu venue vao moi bang so sanh</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>data-bug</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>GHI NHAN (no ky thuat u50 #2, muc CAO)</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>probe xac minh offset tren 2 token + va tai ingest</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>L-31</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>lessons_learned.md rev.1</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Tong hop/dien giai tu tai lieu cu = vung rui ro cao: moi entry phai trace ve cau chu nguon (dinh nghia lay tu yaml/reference, khong tu tri nho dien giai); so lieu khong co trong nguon = khong viet; thuat ngu he thong (M1/M2/ten signal) dung dung nghia goc, khong tai dinh nghia. L-09 ap cho ca tai lieu, khong rieng fire</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>process</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>GHI NHAN</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>moi consolidation sau nay kem bang trace entry-nguon khi operator yeu cau kiem</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>L-32</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
           <t>BANK</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Backfill save nhầm file (_NEW suffix) do file gốc bị lock trong Excel — INDEX vẫn trỏ tên cũ → case_daily ghi vào file cũ (4 dòng) thay vì canonical (35 dòng). Fix: sau bất kỳ backfill nào, verify INDEX trỏ đúng canonical; canonical phải có đúng tên gốc.</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>process/rule</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>GHI NHAN</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>thêm bước verify file name + row count vào checklist sau backfill</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>L-33</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>BANK</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
         <is>
           <t>fn=1 fallback (Zone-A-agg) chỉ dành cho cột taker_buy_pct — KHÔNG mượn sang gLSR/pos_r/acc_r. Metric ratio phải đến từ export CSV hoặc để TRỐNG + comment, không ghép chéo metric. Guard bằng assert EXPORT_COL_MAP tại import time trong case_daily.py.</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr">
+      <c r="E37" t="inlineStr">
         <is>
           <t>rule</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr">
+      <c r="F37" t="inlineStr">
         <is>
           <t>GHI NHAN</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr">
+      <c r="G37" t="inlineStr">
         <is>
           <t>assert đã vào case_daily.py dòng sau FORMULA_COLS</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>L-34</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>CASE_BANK_NEW.xlsx (an 30/07), fix da commit</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>PermissionError khi save xlsx → RAISE RuntimeError ngay, cam silent-save sang ten khac (_NEW suffix). Ten file khac = INDEX tro sai = case_daily ghi nham → data bi pha vo im lang. Fix: close xlsx roi retry</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>process/rule</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>DA VAO case_daily.py (L-34 raise, commit 2026-07-30)</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>backfill script cung phai RAISE neu gap lock (kiem tra backfill.py)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
B5/B6: repo canonical doi ra OneDrive + lessons L-35/L-36/L-37
- CLAUDE.md: bo sung facts canonical path binance-bot-signals
- agent_log.md: session 31/07 B0-B6 ghi du ket qua so
- CASE_INDEX.xlsx: append L-35/L-36/L-37 (37 lessons tong)
- lessons_learned.md: regenerate rev.3 (37 bai hoc)
- Scripts: _task_run_replay_new, _task_scp_bundles, probes
</commit_message>
<xml_diff>
--- a/docs/case_files/CASE_INDEX.xlsx
+++ b/docs/case_files/CASE_INDEX.xlsx
@@ -990,7 +990,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H38"/>
+  <dimension ref="A1:H41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2313,6 +2313,117 @@
       <c r="G38" t="inlineStr">
         <is>
           <t>backfill script cung phai RAISE neu gap lock (kiem tra backfill.py)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>L-35</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>binance-bot-signals P0 regression suite</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Bo calib (12 file _result.txt + GATE dict + replay.py) phai song trong git cung voi code — da dung, ghi nhan de giu. Quy tac: moi repo moi can regression suite commit ngay tu dau, khong de calib file ngoai version control. Loi that nhat la khi calib tach khoi code: code duoc update ma calib cu → false pass / false fail.</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>process/rule</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>GHI NHAN</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>moi repo moi commit regression suite cung voi code trong 24h dau — khong phan tach calib khoi git</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>L-36</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>P0 gate session 31/07 (TAG/BTW reconstruct)</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Tai tao data file phai test bang suite nguyen ban (replay.py goc tu git), KHONG tu viet harness moi. Harness tu viet dan den 3 assertion sai: (1) AKE lsr_accum: viet fires_in thay vi never_in; (2) BASED crowd_flush: viet fires_in thay vi never_in; (3) BULLA pos_rerate: dung file tai tao (pos 07-20=1.75) thay vi file goc (1.99). An: bao 40/43 gia, mat thoi gian debug. Fix: dung replay.py goc → 43/43 PASS.</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>process/rule</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>GHI NHAN</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>quy trinh tai tao data: viet file → chay replay.py goc tu git → PASS truoc khi commit bat ky thu gi</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>L-37</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>B0 bundle backup 4 repo (31/07)</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Repo chi local (khong remote git server) = single point of failure — mot loi o dia hay OneDrive deauth mat het. Giai phap toi thieu: git bundle → SCP len VPS /root/archive/ trong vong 24h tao repo, sau do bundle lai tai moi milestone lon. Da ap 4 repo ngay 31/07: binance-bot-signals, whale_data, Check onchain, Whales_scan. Repo OneDrive them an: file-lock + single-copy = combo sinh an (CASE_BANK_NEW, L-34).</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>rule</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>DA VAO — bundle 4 repo len VPS /root/archive/ ngay 31/07</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>moi repo moi phai co bundle tren VPS trong 24h; nhac lai tai moi milestone lon</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
B4 mo lai + calib-hai-bo + L-38
- CLAUDE.md: calib chi doc tu repo docs/case study/, cam dung loose u50_data
- CASE_INDEX.xlsx: append L-38 (4 nguon 4 so = quy uoc canonical phai ton tai truoc)
- lessons_learned.md: regenerate rev.4 (38 bai hoc)
- proposals/ratio_daily_canonical_20260731.md: de xuat keep-last canonical cho lsr_pos_r
- Probes: derived_1h def, B2 diff 12, B0 verify, B4 canonical, rename loose
</commit_message>
<xml_diff>
--- a/docs/case_files/CASE_INDEX.xlsx
+++ b/docs/case_files/CASE_INDEX.xlsx
@@ -990,7 +990,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H41"/>
+  <dimension ref="A1:H42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2424,6 +2424,43 @@
       <c r="G41" t="inlineStr">
         <is>
           <t>moi repo moi phai co bundle tren VPS trong 24h; nhac lai tai moi milestone lon</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>L-38</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>BULLA 07-20 (B4 probe — 4 nguon 4 so)</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Mot metric mot ngay ra 4 con so khac nhau (1.75/1.68/1.981/1.99) tu 4 nguon: (1) u50 loose = 1.75 (nguon khong ro, retired); (2) top_pos_1h keep-last 23:00 UTC = 1.6811; (3) derived_1h = 00:00 UTC dau ngay = 1.981; (4) native_1d repo goc = 1.99. Nguyen nhan: quy uoc canonical CHUA TON TAI khi calib duoc viet. He qua: verdict buoc phai chon nguon theo ket luan muon co = vi pham nguyen tac. Fix: quy uoc phai duoc ky TRUOC khi bat ky so nao duoc trich dan vao calib/DAILY. Xem proposals/ratio_daily_canonical_20260731.md cho de xuat keep-last canonical.</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>rule</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>GHI NHAN — proposals/ratio_daily_canonical_20260731.md cho operator ky</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>ky proposals/ratio_daily_canonical_20260731.md truoc khi chay backfill tu ngay 31/07</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
boundary canonical v2: CLAUDE.md + L-39 + lessons rev.5
Task 1: CLAUDE.md FACTS — ratio+OI DAILY = snapshot 00:00 UTC mở ngày D
(derived_1h hiện hành), khớp native_1d 21/21 diff 0%; keep-last 23:xx = EVENTS.
Xóa dòng OI-only cũ, hợp nhất vào một dòng ratio+OI.

Task 2 (rà soát ngược — không cần thay đổi code):
- Zone-A-agg TAG 29/07 glsr=1.6059: avg3(1.7071+1.2978+1.8129)/3 = đúng 00:00 UTC
  (từ freshwatch native_1d). Verdict TAG armed không đổi.
- case_daily fn<6: ghi giá trị CSV (00:00 UTC) + SUSPECT comment — không dùng keep-last.

Task 3: L-39 append CASE_INDEX.xlsx LESSONS + regenerate lessons_learned.md (rev.5, 39 bài).
L-39: "Quy ước boundary phải TEST bằng đối chiếu nguồn (21/21 diff 0%) trước khi
văn bản hóa — proposal v1 hợp lý trên giấy nhưng ngược 180° với thực nghiệm;
n=1 suy luận đẹp vẫn phải qua n=21."

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/case_files/CASE_INDEX.xlsx
+++ b/docs/case_files/CASE_INDEX.xlsx
@@ -990,7 +990,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H42"/>
+  <dimension ref="A1:H43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2461,6 +2461,43 @@
       <c r="G42" t="inlineStr">
         <is>
           <t>ky proposals/ratio_daily_canonical_20260731.md truoc khi chay backfill tu ngay 31/07</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>L-39</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>proposal v2 (31/07) — boundary canonical</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Quy ước boundary phải TEST bằng đối chiếu nguồn (21/21 diff 0%) trước khi văn bản hóa — proposal v1 hợp lý trên giấy nhưng ngược 180° với thực nghiệm; n=1 suy luận đẹp vẫn phải qua n=21.</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>rule</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>GHI NHAN — proposal v2 ký 31/07, CLAUDE.md updated</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>trước khi văn bản hóa quy ước metric nào: test &gt;= 21 điểm thực nghiệm đối chiếu nguồn</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
﻿L-40: blast-radius env + lessons rev.6 (40 bai)
L-40: Chot chan cap may co blast radius cap may - truoc khi gat cong tac
dung chung (env/key/config toan cuc), bat buoc liet ke MOI consumer hop le;
rang buoc nham vao agent phai dat o tang hep nhat du dung (per-process wrapper),
khong dat tang chung.
Bang chung: bot fresh wallets chet 3 ngay (31/07-02/08), gap data xac nhan.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/case_files/CASE_INDEX.xlsx
+++ b/docs/case_files/CASE_INDEX.xlsx
@@ -990,7 +990,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H43"/>
+  <dimension ref="A1:H44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2498,6 +2498,43 @@
       <c r="G43" t="inlineStr">
         <is>
           <t>trước khi văn bản hóa quy ước metric nào: test &gt;= 21 điểm thực nghiệm đối chiếu nguồn</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>L-40</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>NANSEN_KEY_LOCKED blast-radius (02/08) — bot fresh wallets</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Chốt chặn cấp máy có blast radius cấp máy — trước khi gạt công tắc dùng chung (env/key/config toàn cục), bắt buộc liệt kê MỌI consumer hợp lệ; ràng buộc nhắm vào agent phải đặt ở tầng hẹp nhất đủ dùng (per-process wrapper), không đặt tầng chung. Bằng chứng: bot fresh wallets chết 3 ngày (gap 31/07–02/08) vì NANSEN_API_KEY rename sang NANSEN_KEY_LOCKED — automated job \FreshWatch không đọc được key.</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>rule</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>DA SUA — run_daily_wrapper.py (02/08); FreshWatch task updated</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>trước khi rename/remove bất kỳ env/key/config toàn cục: grep MỌI consumer (scheduled task + code), sửa wrapper per-process trước khi rename</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
L-42 kho ownership archetype + playbook sync
L-42: IDOL/TAG/BANK — kho spot MM phan loai theo SO HUU (A muon/B unlock/C tu mua).
  Scope notes them C8 cho L-05/L-06/L-07 trong LESSONS sheet.
  lessons_learned.md regen: 42 bai hoc (L-01 → L-42).

analysis_playbook.md: tao moi v0.1 — 6 lop I-VI voi L-42 patches ap vao III.2/III.3/VI.3:
  - III.2: GATE L-42 truoc ma tran M2 (Loai A → THONG DIEP, khong vao bang chung)
  - III.3: shape dep Loai A = tin hieu re, chi tin khi song sot >=X ngay
  - VI.3: checkbox kho Loai A hoi day = thu mua tra no kho = campaign da khep

mm_econ_v0.md: them cot mm_archetype + kho_nguon vao M1/Extended table.
  IDOL=A, BANK=lai A+B, TAG=nghi A; PnL spot ha nhan "unverified inference".
  PENDING K3 sell-side IDOL + BR kho 6% + BANK T+30 09/08.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/case_files/CASE_INDEX.xlsx
+++ b/docs/case_files/CASE_INDEX.xlsx
@@ -1047,7 +1047,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H45"/>
+  <dimension ref="A1:H46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1073,6 +1073,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1299,6 +1300,11 @@
           <t>token dinh bai nay vao SO DEN trong MM_BOOK</t>
         </is>
       </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>[Pham vi L-42]: Loai B/C — withdrawal gan dinh = bang chung phan phoi THAT. Loai A — withdrawal la dao cu, khong vao bang chung; chuyen sang doc theo L-42.</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="15" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
@@ -1336,6 +1342,11 @@
           <t>nguong nhap: V_14d &gt;= 2x withdrawal moi coi la 'co the gom tren venue'</t>
         </is>
       </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>[Pham vi L-42]: Ap dung khi kho xac dinh duoc Loai B hoac C. Loai A — V_venue phan xu 'mua' hay 'hang co san' khong con nghia (hang KHONG thuoc MM); chuyen sang L-42.</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="15" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
@@ -1373,6 +1384,11 @@
           <t>neu BR keo that: doi chieu chot 1+2 co bao truoc khong</t>
         </is>
       </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>[Pham vi L-42]: Ap dung khi xac nhan Loai B/C (kho that). Loai A — kho len san = dao cu chuan bi dan, khong phai leg keo; endgame la round-trip tra no. Doc L-42 truoc L-07.</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="15" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
@@ -2629,6 +2645,48 @@
       <c r="G45" t="inlineStr">
         <is>
           <t>verify vong tu nhien: export sang 04/08 phai ra fn=6 cho ngay 03/08. Neu PASS → dong an. Quy tac: khong bao gio generate D truoc 00:05 UTC D+1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>L-42</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>IDOL/TAG/BANK — kho spot MM: phan loai theo SO HUU truoc khi doc on-chain</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Kho spot cua MM khong tu no la 'hang se xa' — ham muc tieu phu thuoc SO HUU kho. Phan 3 loai TRUOC khi doc bat ky transfer nao: LOAI A (kho MUON tu team — khong gia tri voi MM; P&amp;L 100% o perp; moi deposit/withdrawal la THONG DIEP nhung nguoi doc on-chain, khong phai bang chung; endgame kho round-trip nguyen dai; dong co DAP GIA hau campaign de mua lai tra no kho — canh kho hoi day o day). LOAI B (kho unlock/dau tu — so huu that, cost thap; doanh thu phai hien thuc hoa; neo lich unlock; deposit-len-san &lt;=48h sau ngay unlock = tell hang nhat — BANK 17/07-&gt;18/07). LOAI C (tu bo tien mua tai cho — conviction that, cost basis = floor co nghia, khong deadline; loai duy nhat 'di cung thuyen' duoc). Tell phan loai: (1) NGUON kho — deployer/team wallet = nghi A; vesting contract dung lich = B; gom le nhieu nguon dai han = C; (2) nhip voi lich unlock; (3) hanh vi kho HAU DINH — round-trip nguyen = A, ban that = B; (4) do 'dien' cua transfer — chia may deu + Sent=0 trung bay = tin hieu re, nghi A. Bang chung: IDOL 3 man mot dao cu (8% vao 03-05/07 -&gt; rut 273M staging shape 13 vi -&gt; redeposit 102M) trong khi ket that o perp ~$1.2-1.8M; TAG 90B round-trip May-&gt;Jul; BANK chan unlock ban that (lai A+B); AKE 'perp vol 70x spot — spot la can gat'.</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>rule</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>OPERATOR KY 04/08</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>(a) cot mm_archetype{A/B/C/lai} + kho_nguon cham hoi to 12 case + case song; (b) BR kho 6% trace nguon = viec phan loai dau tien — neu team wallet -&gt; Loai A -&gt; cu flush gLSR 03/08 doc lai duoi anh sang 'dao cu man hai'; (c) moi dong PnL spot chua co sell-side xac nhan ha nhan 'unverified inference' (IDOL 111M, BANK $12-28M); (d) K3 sell-side Pancake IDOL van la test phan xu — PENDING.</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Ap dung cho tat ca case co transfer on-chain. Cap nhat cho L-05/L-06/L-07: scope = Loai B/C; Loai A doc theo L-42 truoc.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
TUT doctrine: two-legged kho + duration scaling
U1: Sửa án nhãn — 08-05 = HARVEST-INTO-STRENGTH / GHẾ-RỜI LẦN 2
    (giá +33%, pos_r −48%, gLSR GIẢM). KHÔNG phải L-26.
    Chốt ③ convention: close-to-close, không VWAP.
    Files: tut_t30_analysis + mm_econ_tut_forward interim note.

U2: CASE_TUT.xlsx — 3 EVENTS (08-05/06/07), thesis_1line → HAI CHAN KHO,
    TRIGGERS + Cửa B pattern.

U3: CASE_INDEX.xlsx LESSONS — L-44(a) kết thúc campaign = kho không phải perp,
    L-45(b) duration scaling. L-43 slot giữ cho operator.

U4: Playbook VII.4 thêm ĐIỀU KIỆN KẾT THÚC CAMPAIGN, VII.5 ghế-rời vs kết thúc,
    VII.7 Q4 build-window, VII.8 duration scaling table.

U5: VII.8 duration scaling n=4 draft (BANK/IDOL/CLO/TUT).

U6: Handover TUT section: sửa nhãn + 7-chốt 08/08 + kho/vol ~50%.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/case_files/CASE_INDEX.xlsx
+++ b/docs/case_files/CASE_INDEX.xlsx
@@ -1047,7 +1047,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H46"/>
+  <dimension ref="A1:H48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2687,6 +2687,60 @@
       <c r="H46" t="inlineStr">
         <is>
           <t>Ap dung cho tat ca case co transfer on-chain. Cap nhat cho L-05/L-06/L-07: scope = Loai B/C; Loai A doc theo L-42 truoc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>L-44</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>L-44(a) DIEU KIEN KET THUC CAMPAIGN: Loai A (kho-muon) = ghe-roi perp la het. Loai B/C (unlock/tu-mua) = ghe-roi perp la CHUYEN PHA — ket thuc that khi kho/vol ≤10% (Cua A) hoac Cua B kich hoat (short-hedge). TUT: pos_r crash 08-05 (−48%) = GHE-ROI LAN 2 (HARVEST-INTO-STRENGTH), KHONG phai L-26, campaign van tiep tuc.</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>TUT</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>DRAFT</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>L-45</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>L-45(b) DURATION SCALING: Thoi luong campaign ty le thuan voi build_window va kho_size. Tham khao draft n=4: BANK (build ~17d, Loai B) → campaign D+17; IDOL (build ~7d, Loai A partial) → D+11; TUT (build 13d, Loai C) → D+16+ ongoing. CLO TBD. Hypothesis: dai build = dai campaign; chua du n de calib chinh xac.</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>TUT/BANK/IDOL/CLO</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>DRAFT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
CASE_HEI cold-start: data collect + case file + report
H0-H6 probes + CASE_HEI.xlsx (540 DAILY rows, 7 sheets, L-32 PASS).
Collect report _collect_hei_20260808.md. CASE_INDEX + INDEX.md cập nhật.
Status=COLD_START PENDING. GOM-A 1 fire (08-01, CHƯA KÝ). LSR 31 rows persisted.
L-23 depth shot #2 MISSING. Contract unconfirmed. DỪNG chờ duyệt.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/case_files/CASE_INDEX.xlsx
+++ b/docs/case_files/CASE_INDEX.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -50,6 +50,9 @@
       <name val="Arial"/>
       <b val="1"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="6">
@@ -107,7 +110,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -129,6 +132,7 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -494,7 +498,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K12"/>
+  <dimension ref="A1:K13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -523,6 +527,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1033,6 +1038,59 @@
       <c r="K12" s="4" t="inlineStr">
         <is>
           <t>leading indicator cua nhau</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>CASE_HEI.xlsx</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>HEI</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>COLD_START — PENDING</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>cold-start perp+spot, spike events 05-29/08-05/08-06</t>
+        </is>
+      </c>
+      <c r="E13" s="9" t="inlineStr">
+        <is>
+          <t>COLD_START</t>
+        </is>
+      </c>
+      <c r="F13" s="9" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="G13" s="9" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="H13" s="9" t="inlineStr">
+        <is>
+          <t>duyệt operator</t>
+        </is>
+      </c>
+      <c r="I13" s="9" t="inlineStr"/>
+      <c r="J13" s="9" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="K13" s="9" t="inlineStr">
+        <is>
+          <t>cold-start 08-08; contract unconfirmed; L-23 2nd depth MISSING</t>
         </is>
       </c>
     </row>
@@ -1073,7 +1131,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
CASE_BANANAS31: cold-start pack (B-0→B-7)
build_case.py: reusable builder refactor từ HEI patch (GOM copy verbatim)
B-1: 503 DAILY rows 2025-03-23→2026-08-07, 50 cols (43 HEI + 7 B-2 diagnostic)
LSR 68 ngày (fresh 30d + freshwatch Jun-Jul); OI/funding/klines đầy đủ
B-2: flag_dist_wall=57d, flag_knife_crowd=9d; pos_r slope ↑ dù giá dump -80% ATH
B-3: 91 dump days ret≤-5%; ATH 0.0373 (2025-07-10); vol≥8x: 31 ngày
B-4: ALPHA_21 fullyDelisted=True; depth snap#1 13:09 UTC Bid=$70k Ask=$49k
B-5: contract 0x3d4f0513...a760 BSC verified via BAPI; BscScan NOTOK CẦN OP
B-6: freshwatch 2026-06+07 có; gom_scan/screen_thresholds: sạch
GOM-A: 25 fires (Jun-Aug 2026); GOM-B: 0; L-32 PASS

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/case_files/CASE_INDEX.xlsx
+++ b/docs/case_files/CASE_INDEX.xlsx
@@ -498,7 +498,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K13"/>
+  <dimension ref="A1:L14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -527,7 +527,15 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
+    <row r="3">
+      <c r="A3" s="9" t="n"/>
+      <c r="B3" s="9" t="n"/>
+      <c r="C3" s="9" t="n"/>
+      <c r="D3" s="9" t="n"/>
+      <c r="E3" s="9" t="n"/>
+      <c r="F3" s="9" t="n"/>
+      <c r="G3" s="9" t="n"/>
+    </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1091,6 +1099,47 @@
       <c r="K13" s="9" t="inlineStr">
         <is>
           <t>cold-start 08-08; contract unconfirmed; L-23 2nd depth MISSING</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>CASE_BANANAS31.xlsx</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>BANANAS31</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>COLD_START — PENDING</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="inlineStr">
+        <is>
+          <t>Alpha fullyDelisted, dump -80% ATH, pos_r~6.7 (BTW/phan phoi?)</t>
+        </is>
+      </c>
+      <c r="E14" s="9" t="inlineStr">
+        <is>
+          <t>COLD_START</t>
+        </is>
+      </c>
+      <c r="F14" s="9" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="G14" s="9" t="inlineStr"/>
+      <c r="H14" s="9" t="inlineStr"/>
+      <c r="I14" s="9" t="inlineStr"/>
+      <c r="J14" s="9" t="inlineStr"/>
+      <c r="K14" s="9" t="inlineStr">
+        <is>
+          <t>ALPHA_21 | contract 0x3d4f...a760 BSC | cold-start 07/08/2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
lessons: L-46/47/48 BANANAS31 (operator signed 09/08)
- CASE_INDEX.xlsx LESSONS sheet: rows 49/50/51 = L-46/47/48
  L-46 ARM: Video vs Photo (pos_r level != BTW alone; 3-derivative check)
  L-47 ARM: dong ho cum — BTW build co expiry (BANANAS31 cum #4 Aug-Oct/26)
  L-48 DATA: fullyDelisted Alpha → ABSTAIN taker_alpha (confirmed IDOL+BANANAS31)
- lessons_learned.md: regen 47 lessons L-01→L-48 (L-43 gap = never written)
- Q1/Q2/Q3 learning path check: PASS (INDEX→playbook→lessons→case)
- Task/probe scripts archived: scripts/archive/

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/case_files/CASE_INDEX.xlsx
+++ b/docs/case_files/CASE_INDEX.xlsx
@@ -498,7 +498,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L14"/>
+  <dimension ref="A1:K14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1154,7 +1154,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H48"/>
+  <dimension ref="A1:H51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2847,6 +2847,117 @@
       <c r="E48" t="inlineStr">
         <is>
           <t>DRAFT</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="9" t="inlineStr">
+        <is>
+          <t>L-46</t>
+        </is>
+      </c>
+      <c r="B49" s="9" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="C49" s="9" t="inlineStr">
+        <is>
+          <t>CASE_BANANAS31 + CASE_HEI</t>
+        </is>
+      </c>
+      <c r="D49" s="9" t="inlineStr">
+        <is>
+          <t>Video vs Photo: hai hồ sơ pos_r cao nhưng ý nghĩa khác nhau. "Video" (CASE_HEI) = build thật: pos_r vừa phải, đồng-bộ giá, ít dist_wall. "Photo" (CASE_BANANAS31) = snapshot đẹp nhưng static: pos_r=6.7 RẤT CAO nhưng sign-corr Δpos_r vs ret_1d ~50% (47.7% opposite) — pos_r KHÔNG predict giá. Thêm: dist_wall_day=57/503 (11.3%), knife_crowd=9 ngày — dấu MM đang bán vào pump. Kết luận: pos_r level đơn độc KHÔNG phân biệt được BTW vs phân phối. Cần 3 đạo hàm: level + slope + sync. Xem Phụ lục A.5. Nguồn: CASE_BANANAS31 phân tích 08-09/08/2026 · ký 09/08 · đối chứng: CASE_HEI.xlsx</t>
+        </is>
+      </c>
+      <c r="E49" s="9" t="inlineStr">
+        <is>
+          <t>ARM</t>
+        </is>
+      </c>
+      <c r="F49" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="G49" s="9" t="inlineStr">
+        <is>
+          <t>Khi pos_r &gt;5: check sign-corr Δpos_r vs ret_1d (30d OLS). &lt;55% → Photo → TRACKING-passive. Không vào setup cho đến đồng hồ cụm trigger (xem L-47). Implement: build_case.py đã in OLS slope + sign-corr.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="9" t="inlineStr">
+        <is>
+          <t>L-47</t>
+        </is>
+      </c>
+      <c r="B50" s="9" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="C50" s="9" t="inlineStr">
+        <is>
+          <t>CASE_BANANAS31</t>
+        </is>
+      </c>
+      <c r="D50" s="9" t="inlineStr">
+        <is>
+          <t>Đồng hồ cụm: Build-into-weakness không kéo dài vô tận. BANANAS31 pump cluster: Jun/Aug/Oct 2026 [n=3 inference từ vol spikes ≥8×med14]. Build cụm #3 từ 06/2026 → đồng hồ ~60-90 ngày → cụm #4 dự kiến Aug-Oct/26. Nếu không có ignite (gLSR≤0.7 + pos rebuild ≥3d) trong cửa sổ → build failed → MM exit. Hiện tại gLSR=1.20 &gt; ngưỡng ignite 1.1 → block entry (crowd đã long hết). Verdict NO_SETUP — TRACKING-passive. Nguồn: CASE_BANANAS31 · ký 09/08</t>
+        </is>
+      </c>
+      <c r="E50" s="9" t="inlineStr">
+        <is>
+          <t>ARM</t>
+        </is>
+      </c>
+      <c r="F50" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="G50" s="9" t="inlineStr">
+        <is>
+          <t>Mỗi case BTW: ghi ngày dự kiến đồng hồ cụm tiếp theo. Theo dõi: gLSR drop về ≤0.7 (lý tưởng) hoặc ≤0.9 (cảnh báo). Nếu hết cửa sổ không trigger → escalate INVALIDATE check.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="9" t="inlineStr">
+        <is>
+          <t>L-48</t>
+        </is>
+      </c>
+      <c r="B51" s="9" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="C51" s="9" t="inlineStr">
+        <is>
+          <t>CASE_BANANAS31 + CASE_IDOL</t>
+        </is>
+      </c>
+      <c r="D51" s="9" t="inlineStr">
+        <is>
+          <t>fullyDelisted Alpha → ABSTAIN taker_alpha. Klines[9]==klines[5] trên BAPI khi fullyDelisted=True (taker column = close price, không phải real taker). Đã confirm: IDOL (ALPHA_223, L-43 context) + BANANAS31 (ALPHA_21). Rule chốt: IF offline=True OR offsell=True OR fullyDelisted=True → taker_alpha=NaN, flag=ABSTAIN. Áp dụng ngược cho mọi case đang mở có Alpha token. Nguồn: CASE_BANANAS31 + CASE_IDOL · ký 09/08</t>
+        </is>
+      </c>
+      <c r="E51" s="9" t="inlineStr">
+        <is>
+          <t>DATA</t>
+        </is>
+      </c>
+      <c r="F51" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="G51" s="9" t="inlineStr">
+        <is>
+          <t>Khi collect Alpha mới: check fullyDelisted trước khi parse klines[9]. Script build_case.py đã implement ABSTAIN block. Audit retrospective: CASE_TUT/BR/CLO — check Alpha status.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
cold-start CASE_TST: 545 DAILY rows, A.5 bảng, đăng ký INDEX
- CASE_TST.xlsx: 7 sheets, 545 DAILY (2025-02-09→2026-08-07), 50 cols
- ATH listing day 0.2252, drawdown -94%, vol spike 07/08 27x
- gLSR 1.54→2.36 (42d window), GOM-A 0 fires (A2 fail toàn bộ)
- Funding âm mạnh 04-07/08 (f_avg=-0.00177 ngày 05/08)
- Depth snap #1 00:08 UTC, snap #2 MISSING (chờ ≥04:08)
- Đăng ký CASE_INDEX + INDEX.md
- _collect_tst_20260809.md: report raw + MISSING list

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/case_files/CASE_INDEX.xlsx
+++ b/docs/case_files/CASE_INDEX.xlsx
@@ -528,13 +528,45 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="9" t="n"/>
-      <c r="B3" s="9" t="n"/>
-      <c r="C3" s="9" t="n"/>
-      <c r="D3" s="9" t="n"/>
-      <c r="E3" s="9" t="n"/>
-      <c r="F3" s="9" t="n"/>
-      <c r="G3" s="9" t="n"/>
+      <c r="A3" s="9" t="inlineStr">
+        <is>
+          <t>CASE_TST.xlsx</t>
+        </is>
+      </c>
+      <c r="B3" s="9" t="inlineStr">
+        <is>
+          <t>TST</t>
+        </is>
+      </c>
+      <c r="C3" s="9" t="inlineStr">
+        <is>
+          <t>COLD_START — PENDING</t>
+        </is>
+      </c>
+      <c r="D3" s="9" t="inlineStr">
+        <is>
+          <t>Alpha fullyDelisted, ATH=listing day, -94% drawdown. Massive vol spike 07/08 (+20%, 27x, funding negative). Cau hoi: co luc gom hang khong?</t>
+        </is>
+      </c>
+      <c r="E3" s="9" t="inlineStr">
+        <is>
+          <t>COLD_START</t>
+        </is>
+      </c>
+      <c r="F3" s="9" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="G3" s="9" t="inlineStr"/>
+      <c r="H3" s="9" t="inlineStr"/>
+      <c r="I3" s="9" t="inlineStr"/>
+      <c r="J3" s="9" t="inlineStr"/>
+      <c r="K3" s="9" t="inlineStr">
+        <is>
+          <t>ALPHA_87 | BSC 0x86bb94...666429 | cold-start 08/08/2026</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">

</xml_diff>

<commit_message>
AGT cold-start pack: CASE_AGT.xlsx 445d + A-0 build_case patch + depth snap ×2
- CASE_AGT.xlsx: 7 sheets, 445 DAILY rows (2025-05-20→2026-08-07), 50 cols, GOM-A=0
- build_case.py: parametrize metadata dynamic (A-0a); fix lsr/spot key mismatch; A-0b guards
- Depth snap #1 08:44 UTC ratio=0.524 ask-heavy; snap #2 13:21 UTC ratio=1.10 bid-slight
- Register: CASE_INDEX row + INDEX.md
- archive: 5 AGT probe scripts

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/case_files/CASE_INDEX.xlsx
+++ b/docs/case_files/CASE_INDEX.xlsx
@@ -498,7 +498,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K14"/>
+  <dimension ref="A1:K16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1172,6 +1172,79 @@
       <c r="K14" s="9" t="inlineStr">
         <is>
           <t>ALPHA_21 | contract 0x3d4f...a760 BSC | cold-start 07/08/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t>CASE_AGT.xlsx</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>AGT</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>COLD_START — PENDING</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>Alaya Governance Token. Perp onboard 2025-05-20, ATH=2025-05-27 (0.034016). Drawdown -56%. 19 vol spikes &gt;=8x. gLSR luon &gt;1.5 (retail crowded long). GOM-A 0 fires. Cau hoi: co luc gom, dang o pha nao?</t>
+        </is>
+      </c>
+      <c r="E15" s="9" t="inlineStr">
+        <is>
+          <t>COLD_START</t>
+        </is>
+      </c>
+      <c r="F15" s="9" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="G15" s="9" t="inlineStr"/>
+      <c r="H15" s="9" t="inlineStr"/>
+      <c r="I15" s="9" t="inlineStr"/>
+      <c r="J15" s="9" t="inlineStr"/>
+      <c r="K15" s="9" t="inlineStr">
+        <is>
+          <t>ALPHA_191 | BSC 0x5dbde81...e274 | cold-start 08/08/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>FFUSDT</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>FF</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>COLD_START — AUDIT PENDING</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>ALPHA_398</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Bot báo gom ~$2M trên perp — tái lập số, ba phương pháp §3 độc lập</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
COOKIE audit-collect 20260809: C-0→C-8 + CASE_COOKIE.xlsx + CASE_INDEX đăng ký
Pipeline đầy đủ: truy alert GOM-C (n=1, Q1=$0, VWAP=$0.00774), LSR 44d,
perp/spot 579r, fund 500rec, OI 30d. §3 ba phương pháp: Q1_chain=$0,
Q2_net=+$238K, Q3=$993K-$2.98M. Rechấm GOM-C 08-03: C2✓C3✓ d_pos FAIL.
ATH-97.9%, oi_cycle=0.289, hedge_struct=90%. Depth snap#1 01:50 UTC ratio=1.49.
CASE_COOKIE.xlsx 7 sheets 138KB. CASE_INDEX row 17. DỪNG chờ operator verdict.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/case_files/CASE_INDEX.xlsx
+++ b/docs/case_files/CASE_INDEX.xlsx
@@ -498,7 +498,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K16"/>
+  <dimension ref="A1:K17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1245,6 +1245,53 @@
       <c r="F16" t="inlineStr">
         <is>
           <t>Bot báo gom ~$2M trên perp — tái lập số, ba phương pháp §3 độc lập</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>CASE_COOKIE.xlsx</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>COOKIE</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>OPEN — audit-collect complete, awaiting operator verdict</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>GOM-C fire 08-03; pump pattern; ATH-97.9%; OI $1.1M</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>COLD_START</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>depth snap #2 ≥05:50 UTC</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>fullyDelisted=True; Q1=0(chain); oi_cycle=0.289; VWAP=$0.00774</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
BR3 BROCCOLIF3B audit-collect: BR3-0→BR3-8 PASS
- BR3-0: two-broccoli identity lock (F3B vs 714, distinct baseAssets, PASS)
- BR3-1: LSR 4 endpoints 30d + OI hist, gLSR=4.96-5.98 (short bias cực cao)
- BR3-2: 507 perp klines full history, CASE_BROCCOLIF3B.xlsx 50cols/7sheets/109KB
- BR3-3: Q1_NET=$4.35M, Q2_net=$640K, Q3=N/A, VWAP=+9.97%, GOM-C 1 ngày PROVISIONAL
- BR3-4: ATH-89%, ignition đã xảy ra 07-22/27, flag_hedge_struct=63.3%, oi_cycle=0.37
- BR3-5: NOT Alpha token, depth snap#1 mid=$0.006935 ratio=1.585 bid-heavy, gate>=04:45
- BR3-6: sổ chéo — first case, F3B/714 tách biệt trong FW, 0 tiền sử gom_scan
- BR3-7: 6/6 PASS
- BR3-8: CASE_INDEX row18 OPEN COLD_START, INDEX.md regen
DUNG cho doc — khong verdict

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/case_files/CASE_INDEX.xlsx
+++ b/docs/case_files/CASE_INDEX.xlsx
@@ -498,7 +498,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K17"/>
+  <dimension ref="A1:K18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1292,6 +1292,51 @@
       <c r="K17" t="inlineStr">
         <is>
           <t>fullyDelisted=True; Q1=0(chain); oi_cycle=0.289; VWAP=$0.00774</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>CASE_BROCCOLIF3B.xlsx</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>BROCCOLIF3B</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>COLD_START</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>COLD_START</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>depth snap#2 &gt;=04:45 UTC 2026-08-10</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>BR3 audit-collect 10/08; two-broccoli confirmed distinct; DUNG cho doc</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
K KOMA audit-collect: K-0→K-8 PASS + GOM-C PROVISIONAL
- K-0: KOMAUSDT identity lock, ALPHA_1 (first Alpha), fullyDelisted=False, no KOMAINU
- K-1: LSR 4 endpoints 30d + OI hist $1.6M→$19.4M (UNCALIBRATED), FW u137
- K-2: 608 klines full history, CASE_KOMA.xlsx 50cols/7sheets/128KB
- K-3: Q1_GROSS=$19M Q1_NET=$8.96M (89% tu FLUSH 08-01), Q2 UNCALIB, VWAP=-28.6%
- K-3: GOM-C PROVISIONAL 2 ngay (07-23, 08-02) — nhap ho so gate 15/08
- K-4: MEGA-PUMP 07-31 +100%/$604M, FLUSH 08-01 -39%/$457M, px-ATH=-92%
- K-5: Alpha ACTIVE, depth snap#1 mid=$0.01391 ratio=2.169, gate>=05:51 UTC
- K-7: 6/6 PASS; K-8: CASE_INDEX row19 OPEN GOM-C PROVISIONAL COLD_START
DUNG cho doc — khong verdict

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/case_files/CASE_INDEX.xlsx
+++ b/docs/case_files/CASE_INDEX.xlsx
@@ -498,7 +498,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K18"/>
+  <dimension ref="A1:K19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1326,17 +1326,63 @@
           <t>2026-08-10</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr">
         <is>
           <t>depth snap#2 &gt;=04:45 UTC 2026-08-10</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
       <c r="K18" t="inlineStr">
         <is>
           <t>BR3 audit-collect 10/08; two-broccoli confirmed distinct; DUNG cho doc</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>CASE_KOMA.xlsx</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>KOMA</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>GOM-C PROVISIONAL</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>COLD_START</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>depth snap#2 &gt;=05:51 UTC; GOM-C gate 15/08</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>ALPHA_1</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>K audit-collect 10/08; pump 07-31 +100%/$604M; OI UNCALIB; GOM-C PROV 07-23+08-02</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
APR audit-collect: A-0→A-8 done, 291 klines, GOM-C 22d PROVISIONAL
- APRUSDT perp-only (not Alpha), onboard 2025-10-23, LSR endpoint all 404
- 291 DAILY rows (2025-10-23→2026-08-09), OI calibrated ($8.26M-$10.92M)
- GOM-C PROVISIONAL 22 ngày (Jun 2→Aug 4), C1 pending
- Q1_NET=$5.20M (89.7%), ATH=-73.45%, div_avg3=1.70 peak 2.16
- Sanity 6/6 PASS, build exit=0 (no guard-câm)
- CASE_INDEX row 20, snap#2 gate ≥07:42 UTC

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/case_files/CASE_INDEX.xlsx
+++ b/docs/case_files/CASE_INDEX.xlsx
@@ -498,7 +498,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K19"/>
+  <dimension ref="A1:K20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1368,13 +1368,11 @@
           <t>2026-08-10</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr">
         <is>
           <t>depth snap#2 &gt;=05:51 UTC; GOM-C gate 15/08</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr"/>
       <c r="J19" t="inlineStr">
         <is>
           <t>ALPHA_1</t>
@@ -1383,6 +1381,55 @@
       <c r="K19" t="inlineStr">
         <is>
           <t>K audit-collect 10/08; pump 07-31 +100%/$604M; OI UNCALIB; GOM-C PROV 07-23+08-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>CASE_APR.xlsx</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>APR</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>GOM-C 22ngay PROVISIONAL</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>COLD_START</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>depth snap#2 &gt;=07:42 UTC; GOM-C C1 gate 15/08</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>N/A (not Alpha)</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>perp-only (not Alpha); onboard 2025-10-23; ATH=$0.75→-73%; GOM-C 22d Jun-Aug; OI calib</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
packet BTW: CASE_BTW.xlsx build + W-0→W-7 analytics + CASE_INDEX row 21
- W-0 án tích: BTW calib#6, DQ cool end 31/07, S5 SUPPRESSED 20/07
- W-1 LSR+OI: 4 endpoints 404, OI UNCALIBRATED $6.6M→$48.8M
- W-2 collect: 67 klines Jun5→Aug10, blowoff 2.0 Aug5-9 ($198M peak)
- W-2b build: exit=0, 66 rows × 50 cols, 5 GOM-A fires (Jun blowoff + Jul)
- W-3 triage: div_avg3=2.37 HIGH_LONG, gLSR=0.80 BEAR, f_avg_3=0.000832 (14× pin) → trigger 0/3
- W-4 lifecycle: phase=BLOWOFF2.0, oi_cycle_pos=0.899, new ATH $0.224 (Aug7)
- W-5 snap1: 08:01 UTC, mid=$0.1988, BID-HEAVY ratio=1.249, snap2 gate ≥12:01
- W-6 sanity: 5/5 PASS (verify-tay exact match, OI flag, div_avg3 consistent)
- W-7 CASE_INDEX: row 21 BTWUSDT COLD_START PENDING

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/case_files/CASE_INDEX.xlsx
+++ b/docs/case_files/CASE_INDEX.xlsx
@@ -498,7 +498,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K20"/>
+  <dimension ref="A1:K21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1415,13 +1415,11 @@
           <t>2026-08-10</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr">
         <is>
           <t>depth snap#2 &gt;=07:42 UTC; GOM-C C1 gate 15/08</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr"/>
       <c r="J20" t="inlineStr">
         <is>
           <t>N/A (not Alpha)</t>
@@ -1430,6 +1428,38 @@
       <c r="K20" t="inlineStr">
         <is>
           <t>perp-only (not Alpha); onboard 2025-10-23; ATH=$0.75→-73%; GOM-C 22d Jun-Aug; OI calib</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>CASE_BTW.xlsx</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>BTW</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>COLD_START — PENDING</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>BLOWOFF2.0 echo; 3-cond trigger 0/3; OI UNCALIBRATED; GOM-C 14d pre-cool</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>WATCH (án tích refresh)</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ON pipeline N-0→N-8: CASE_ON.xlsx 289 DAILY, stage S3, snap1 ASK-HEAVY
ALPHA_444 / ONUSDT. Sanity 5/5 PASS.
- div_avg3=1.41 BULL, gLSR=0.85 BEAR, f_avg_3=0.000385 NOT_PIN
- Stage S3 xa-vung-nho: px -20.5% tu ATH $0.46 (Aug7), dist_wall=22d
- GOM-A 0 fires, GOM-C 3 ngay post-Aug1 (C2 FAIL hom nay)
- Depth snap1 09:02UTC ratio=0.7739 ASK-HEAVY, gate snap2 >=13:02UTC
- CAN OPERATOR: BscScan v2 top holders, Nansen exchange balance

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/case_files/CASE_INDEX.xlsx
+++ b/docs/case_files/CASE_INDEX.xlsx
@@ -498,7 +498,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K21"/>
+  <dimension ref="A1:K22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1460,6 +1460,48 @@
       <c r="F21" t="inlineStr">
         <is>
           <t>2026-08-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>CASE_ON.xlsx</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>DIST_WALL ATH-XẢ; 0 GOM-A; OI UNCALIBRATED; stage S3 xả-vùng-nhớ</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>WATCH (án mới, stage S3 pending confirmation)</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>snap2 &gt;=13:02 UTC; N-4 on-chain CẦN OPERATOR</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>ALPHA_444; onboard 2025-10-24; ATH $0.46 Aug7; 289 DAILY rows; contract=0x0e4f6209...</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
GUA audit-collect G-0→G-8: CASE_GUA.xlsx 231 rows, snap2 pending
SUPERFORTUNE (ALPHA_483): crowd-trap structure — div_avg3=0.41 BEAR,
gLSR=2.87 VERY BULL, ATH $1.70 -97.7%, pump TODAY +54.92% 17.96×.
GOM-A/B COLD; GOM-D draft D1+D3+D4+D5 PASS (staged-pump DNA lịch sử).
CẦN OPERATOR: on-chain top holders + wallet crossref ON/BTW/AGT.
CASE_INDEX row 23. Snap2 pending ≥15:50 UTC.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/case_files/CASE_INDEX.xlsx
+++ b/docs/case_files/CASE_INDEX.xlsx
@@ -498,7 +498,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K22"/>
+  <dimension ref="A1:K23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1502,6 +1502,53 @@
       <c r="K22" t="inlineStr">
         <is>
           <t>ALPHA_444; onboard 2025-10-24; ATH $0.46 Aug7; 289 DAILY rows; contract=0x0e4f6209...</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>CASE_GUA.xlsx</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>GUA</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>crowd-trap; div_avg3=0.41 BEAR; gLSR=2.87 VERY BULL; 0 GOM-A; OI calib $5.4M; ATH $1.70 -97.7%; pump TODAY +54.92%</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>WATCH (án mới, pump in-progress → DỪNG chờ đọc)</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>snap2 ≥15:50 UTC; G-4 on-chain CẦN OPERATOR; G-5 snap1 BID-HEAVY 1.25</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>ALPHA_483</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>SUPERFORTUNE; BSC onboard 2025-12-21; ATH $1.70 May25; 231 DAILY rows; contract=0xa5c8e151...</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ĐÓNG P0+GUARD-CÂM: md5=a5a929dc IDENTICAL; L-49/50/51 vào CASE_INDEX; C1 draft → handover
- md5 closed chapters IDENTICAL post-cron 01:25 UTC 08-11 → §8.2 PASS
- P0 và GUARD-CÂM đóng chính thức
- CASE_INDEX.xlsx: L-49 (validate_gom_state), L-50 (P0 root cause slope boundary), L-51 (C1 spec stale comments)
- docs/handover/c1_spec_draft_20260811.md: draft C1 thành văn gửi ANALYSIS [CHỜ XÁC NHẬN 0.09/1.3×]
- agent_log: đính chính audit lỗi (9%≠15% sai — thresholds.yaml có 0.09 đúng)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/case_files/CASE_INDEX.xlsx
+++ b/docs/case_files/CASE_INDEX.xlsx
@@ -1563,7 +1563,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H51"/>
+  <dimension ref="A1:H54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -3367,6 +3367,117 @@
       <c r="G51" s="9" t="inlineStr">
         <is>
           <t>Khi collect Alpha mới: check fullyDelisted trước khi parse klines[9]. Script build_case.py đã implement ABSTAIN block. Audit retrospective: CASE_TUT/BR/CLO — check Alpha status.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>L-49</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>GUARD-CÂM / ALL tokens</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>save_state() fail-open: ghi state.json không kiểm tra invariants → state corrupt không bị bắt. Sửa: validate_gom_state() wired vào save_state() pre-write (4 invariants: open chain ≤3d gap, không open+cooldown đồng thời, vwap_type hợp lệ, cooldown_end ≥ episode_start). Violation → RuntimeError → exit≠0 → Telegram alert (L-44). Commit c3d49e1.</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>GUARD</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>DA VAO gom_scan.py c3d49e1</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>Verify sau SCP: validator không thay đổi write behavior (md5 re-check post manual run)</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>L-50</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>P0 / FFUSDT 2026-08-01</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>P0 root cause: floating-point boundary tại A3 slope_5d = 1.15. FFUSDT 08-01: slope=1.14902 (dist=0.00098 từ ngưỡng). State corrupt xảy ra vì backfill chạy lại trên đoạn đã có chapter, không phải cron viết lại. Incremental mode §8.2 đã xác nhận đúng: md5 closed-chapters IDENTICAL sau cron 01:25 UTC 08-11 (a5a929dcc4ba17f71eb3243146be2314). Vùng-rung probe: A3 có 32 changed-outcome events / 60d / 525 tokens tại ε=0.005. Mốc V4 monitor: MARGINAL-V4 đến 25/08.</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>DONG — md5 PASS 11/08</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>V4 monitor: đếm chain oscillation do A2/A3 marginal qua marginal_hits.csv đến 25/08</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>L-51</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>GOM-C C1 spec / TỔNG HỢP</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Code comments (# 0.15 / # 1.5 trong signals.py) là stale defaults — không phải running values. Running values đến từ thresholds.yaml: breakout_pct=0.09 / oi_mult=1.3 (calibrated cho TUT P0-close). Spec v1.5 số đúng nhưng thiếu 3 điều kiện cấu trúc: (1) range_end=i-5 (14d range kết thúc TRƯỚC 5d build window); (2) OR-check: giá đạt target bất kỳ ngày nào trong 5d; (3) taker check là max(window)&lt;55%, không phải per-day. Bài học: khi spec nói 'X thay Y' trong changelog — luôn trace thresholds.yaml chứ không đọc code comments.</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>SPEC-DRIFT</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>DE XUAT — chờ ANALYSIS ký C1 text ≤14/08</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>ANALYSIS xác nhận số canonical (0.09/1.3× hay 0.15/1.5×) + ký C1 text → operator ký ≤14/08</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sửa comment signals.py + L-51 framing + WARN L-43 gap
- signals.py (binance-bot-signals 4606b86b): # 0.15/1.5 → # 0.09/1.3 (runtime-confirmed)
- CASE_INDEX L-51: framing "comment sai (lying comments = bug), đã sửa commit 4606b86b"
- agent_log: đính chính C1 — không phải "audit nhầm" mà "comment signals.py lệch yaml — comment sai, đã sửa"
- WARN: L-43 MISSING trong LESSONS, L-44/L-45 column mismatch (ngay nhận text thay ngày)
- Probe files: _probe_c1_runtime, _probe_lessons_l43_check, _probe_lessons_structure
- Task files: _task_close_guard_cam_lesson, _task_fix_l51_framing

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/case_files/CASE_INDEX.xlsx
+++ b/docs/case_files/CASE_INDEX.xlsx
@@ -1589,6 +1589,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -3462,7 +3463,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Code comments (# 0.15 / # 1.5 trong signals.py) là stale defaults — không phải running values. Running values đến từ thresholds.yaml: breakout_pct=0.09 / oi_mult=1.3 (calibrated cho TUT P0-close). Spec v1.5 số đúng nhưng thiếu 3 điều kiện cấu trúc: (1) range_end=i-5 (14d range kết thúc TRƯỚC 5d build window); (2) OR-check: giá đạt target bất kỳ ngày nào trong 5d; (3) taker check là max(window)&lt;55%, không phải per-day. Bài học: khi spec nói 'X thay Y' trong changelog — luôn trace thresholds.yaml chứ không đọc code comments.</t>
+          <t>Comment signals.py lệch yaml — comment sai (lying comments = bug), đã sửa commit 4606b86b. Running values từ thresholds.yaml: breakout_pct=0.09 / oi_mult=1.3 (calibrated TUT P0-close). Runtime-confirmed bằng _probe_c1_runtime_20260811.py STEP 1+2. Spec v1.5 '+9%/1.3×' KHỚP thresholds.yaml = ĐÚNG về số. Còn 3 điều kiện cấu trúc thiếu trong spec: (1) range_end=i-5 (14d range kết thúc TRƯỚC 5d build window); (2) OR-check: giá đạt target bất kỳ ngày nào trong 5d; (3) taker check là max(window)&lt;55%, không phải per-day. Bài học: khi spec changelog nói 'X thay Y' → luôn trace thresholds.yaml, không đọc code comments.</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -3472,7 +3473,7 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>DE XUAT — chờ ANALYSIS ký C1 text ≤14/08</t>
+          <t>DA SUA — comment fix 4606b86b + runtime-confirmed 11/08</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">

</xml_diff>

<commit_message>
CASE_CYS.xlsx cold-start: collect C-0→C-8 CYSUSDT 13/08
224 rows Jan01-Aug12. GOM-C Aug07 PROVISIONAL (gate 15/08 pending).
Bốn vân: pos_r −63.5% (giảm), hedge Jul02-18 (17d div<1),
short squeeze Aug05 (acc_r 1.68→0.38), on-chain Solana MISSING.
OI: $12.2M(Jun01)→$7.1M(Aug03)→$23.1M(pump) = phân phối + squeeze.
Perp depth ±2% = $507 với OI $30M → flag wash-test candidate.
Verdict thu thập: C/D staged-pump. DỪNG chờ operator đọc.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/case_files/CASE_INDEX.xlsx
+++ b/docs/case_files/CASE_INDEX.xlsx
@@ -498,7 +498,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K23"/>
+  <dimension ref="A1:K24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1549,6 +1549,43 @@
       <c r="K23" t="inlineStr">
         <is>
           <t>SUPERFORTUNE; BSC onboard 2025-12-21; ATH $1.70 May25; 231 DAILY rows; contract=0xa5c8e151...</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>CASE_CYS.xlsx</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>CYS</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>COLD_START — PENDING</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>GOM audit: gom thật vs staged-pump. Short squeeze Aug04-12 (+438% từ Jun trough). 4 vân: pos_r GIẢM, hedge Jul, squeeze Aug05. CẦN on-chain Solana.</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>COLD_START</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>ALPHA_495 | Solana | collect 13/08/2026 | on-chain CẦN OPERATOR</t>
         </is>
       </c>
     </row>
@@ -1589,7 +1626,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
CASE_AIN.xlsx cold-start: collect AI-0→AI-8 AINUSDT 13/08
Intel operator: 30M token ≈ $2.4M nạp từ 04/08.
224 rows Jan01-Aug12. GOM-D 4/4 PASS. GOM-E 29d hedge PASS.
Deposit taxonomy BLEED. Chain UNKNOWN. 5/5 sanity PASS.
DỪNG chờ đọc _collect_ain_20260813.md.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/case_files/CASE_INDEX.xlsx
+++ b/docs/case_files/CASE_INDEX.xlsx
@@ -498,7 +498,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K24"/>
+  <dimension ref="A1:K25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1586,6 +1586,43 @@
       <c r="K24" t="inlineStr">
         <is>
           <t>ALPHA_495 | Solana | collect 13/08/2026 | on-chain CẦN OPERATOR</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>CASE_AIN.xlsx</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>AIN</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>COLD_START — PENDING</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Deposit intel: 30M token ≈ $2.4M từ 04/08. GOM-D 4/4 PASS, GOM-E PASS 29d hedge. Taxonomy BLEED. Blockchain UNKNOWN. Gate thin $78K/d. CẦN OPERATOR on-chain.</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>COLD_START</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>AI narrative | chain UNKNOWN | collect 13/08/2026 | on-chain CẦN OPERATOR</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
handover: analysis topic close 20260817
- docs/handover/analysis_handover_20260817.md: file đọc thứ nhì (§1 bảng 17 case + §2 học thuyết + §3-§7 spec/infra/pending)
- docs/INDEX.md: thêm dòng handover vào Tầng 1 boot sequence
- docs/analysis_playbook.md v0.3: append §VIII 14 học thuyết phiên 17/08 + cross-ref
- CASE_INDEX.xlsx: sync state AIN→TRACKING-ACTIVE · APR→DISTRIBUTION-WATCH · GUA→S2-WATCH·DIST · BTW→DISTRIBUTION-WATCH · ON→DISTRIBUTION-WATCH·S2-leg3

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/case_files/CASE_INDEX.xlsx
+++ b/docs/case_files/CASE_INDEX.xlsx
@@ -498,7 +498,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K25"/>
+  <dimension ref="A1:S25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -923,7 +923,7 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>du kien CASE-05</t>
+          <t>DISTRIBUTION-WATCH</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
@@ -1397,7 +1397,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>DISTRIBUTION-WATCH</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1444,7 +1444,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>COLD_START — PENDING</t>
+          <t>DISTRIBUTION-WATCH</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1476,7 +1476,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>ACTIVE</t>
+          <t>DISTRIBUTION-WATCH · S2-leg3</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1518,7 +1518,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>ACTIVE</t>
+          <t>S2-WATCH · DISTRIBUTION</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1602,7 +1602,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>COLD_START — PENDING</t>
+          <t>TRACKING-ACTIVE</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">

</xml_diff>

<commit_message>
L-28 am.1 · căn cước bằng giá contract + ledger migration notes
- CASE_INDEX.xlsx LESSONS: append L-28 am.1 (nguồn ngoài neo căn cước = khớp giá contract với perp ≤5×)
- lessons_learned.md: regen từ sheet với header source_md5 + generated_at (L-74)
- ARX/PLAY/AIN/CROSS: ghi chú migration ledger 28/09 (ARX 'arcs' vô hiệu · PLAY kho N/A do contract sai · AIN alive dù offline · CROSS/ONE dup contract)

Nguồn: v28d N1-N3 · classifier v28c pending ANALYSIS ký. KHÔNG sửa whales_config prod.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/case_files/CASE_INDEX.xlsx
+++ b/docs/case_files/CASE_INDEX.xlsx
@@ -10,6 +10,7 @@
     <sheet name="LESSONS" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="MM_BOOK" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="PHAN_VAI" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="CASES" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -1741,7 +1742,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I101"/>
+  <dimension ref="A1:R121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -5300,6 +5301,1097 @@
       <c r="I101" t="inlineStr">
         <is>
           <t>REV10-APPLY</t>
+        </is>
+      </c>
+    </row>
+    <row r="102"/>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>LR_id</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>ve</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>loai</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>support_n</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>counter_n</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>cases_support</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>cases_counter</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>cases_not_applicable</t>
+        </is>
+      </c>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>cases_true_negative</t>
+        </is>
+      </c>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>cases_pending</t>
+        </is>
+      </c>
+      <c r="K103" t="inlineStr">
+        <is>
+          <t>gate_binding</t>
+        </is>
+      </c>
+      <c r="L103" t="inlineStr">
+        <is>
+          <t>evidence_class</t>
+        </is>
+      </c>
+      <c r="M103" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="N103" t="inlineStr">
+        <is>
+          <t>thresholds_signed</t>
+        </is>
+      </c>
+      <c r="O103" t="inlineStr">
+        <is>
+          <t>signed_by</t>
+        </is>
+      </c>
+      <c r="P103" t="inlineStr">
+        <is>
+          <t>signed_date</t>
+        </is>
+      </c>
+      <c r="Q103" t="inlineStr">
+        <is>
+          <t>last_regrade</t>
+        </is>
+      </c>
+      <c r="R103" t="inlineStr">
+        <is>
+          <t>changelog</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>LR-01b</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>pos_r ≥[3] ∧ pin ≥[7d] ∧ |ΔOI 14d| ≤[15%] ∧ px ≤ đáy dải 30d → ×3/120d</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>A-stealth</t>
+        </is>
+      </c>
+      <c r="D104" t="n">
+        <v>2</v>
+      </c>
+      <c r="E104" t="n">
+        <v>0</v>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>BANK:2026-07-19:7e520f40, TUT:2026-08-02:4ab482bc</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>AKE:2026-09-10:92fa9c56, BTW:2026-09-10:ffe6b6de, BTR:2026-09-10:c988194e, 龙虾:2026-09-10:2b727853</t>
+        </is>
+      </c>
+      <c r="K104" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="L104" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="M104" t="inlineStr">
+        <is>
+          <t>HYPOTHESIS</t>
+        </is>
+      </c>
+      <c r="Q104" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="R104" t="inlineStr">
+        <is>
+          <t>2026-09-10 · seed · T1</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>LR-04</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>vol ≥×[8] med14 ∧ ret về ±[10%] nền ≤3d ∧ ≤[45]d trước D0 (bait-probe)</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="D105" t="n">
+        <v>11</v>
+      </c>
+      <c r="E105" t="n">
+        <v>2</v>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>BANK:2026-09-10:7e520f40, TUT:2026-09-10:4ab482bc, AKE:2026-09-10:92fa9c56, BTW:2026-09-10:ffe6b6de, BTR:2026-09-10:c988194e, CAP:2026-09-10:2695bc3f, ON:2026-09-10:4e0e3a7a, HEMI:2026-09-10:4238441f, BULLA:2026-09-10:deb0b268, 龙虾:2026-09-10:2b727853, UAI:2026-09-10:af767473</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>CYS:2026-09-10:af073e64, PROM:2026-09-10:b50b1f68</t>
+        </is>
+      </c>
+      <c r="K105" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="L105" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="M105" t="inlineStr">
+        <is>
+          <t>RETIRED</t>
+        </is>
+      </c>
+      <c r="Q105" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="R105" t="inlineStr">
+        <is>
+          <t>2026-09-10 · seed · T1 · 2026-09-11 · CANDIDATE→RETIRED · counter_n=2≥2</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>LR-05</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>taker_buy &lt;[55%] xuyên markup (≤1 ngày eve)</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="D106" t="n">
+        <v>13</v>
+      </c>
+      <c r="E106" t="n">
+        <v>0</v>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>AKE:2026-09-10:92fa9c56, TUT:2026-09-10:4ab482bc, BANK:2026-09-10:7e520f40, BTW:2026-09-10:ffe6b6de, BTR:2026-09-10:c988194e, CAP:2026-09-10:2695bc3f, ON:2026-09-10:4e0e3a7a, HEMI:2026-09-10:4238441f, BULLA:2026-09-10:deb0b268, 龙虾:2026-09-10:2b727853, UAI:2026-09-10:af767473, CYS:2026-09-10:af073e64, PROM:2026-09-10:b50b1f68</t>
+        </is>
+      </c>
+      <c r="K106" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L106" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="M106" t="inlineStr">
+        <is>
+          <t>RULE-XÁC-NHẬN</t>
+        </is>
+      </c>
+      <c r="N106" t="inlineStr">
+        <is>
+          <t>descriptive:55</t>
+        </is>
+      </c>
+      <c r="O106" t="inlineStr">
+        <is>
+          <t>Tiên</t>
+        </is>
+      </c>
+      <c r="P106" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="Q106" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="R106" t="inlineStr">
+        <is>
+          <t>2026-09-10 · seed · T1 · Tiên ký 10/09</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>LR-06</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>pos_r ↓ ≥25% ∧ OI ↑ ∧ gLSR ↓ = crowd-short-nạp (fuel), không phải MM exit</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>A/D</t>
+        </is>
+      </c>
+      <c r="D107" t="n">
+        <v>1</v>
+      </c>
+      <c r="E107" t="n">
+        <v>1</v>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>TUT:2026-08-02:4ab482bc</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>BANK:2026-07-19:7e520f40</t>
+        </is>
+      </c>
+      <c r="K107" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L107" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="M107" t="inlineStr">
+        <is>
+          <t>HYPOTHESIS</t>
+        </is>
+      </c>
+      <c r="Q107" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="R107" t="inlineStr">
+        <is>
+          <t>2026-09-10 · seed · T1</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>LR-07</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>nạp ≥[50%]/5d ∧ ret ≤−[30%]/5d ∧ plateau ≥[5]d ∧ acc ≥[2] ∧ div_avg3 TĂNG = STAGING (làm giá)</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>B/C</t>
+        </is>
+      </c>
+      <c r="D108" t="n">
+        <v>2</v>
+      </c>
+      <c r="E108" t="n">
+        <v>1</v>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>AKE:2026-09-10:92fa9c56, BTR:2026-09-10:c988194e</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>BANK:2026-07-20:7e520f40</t>
+        </is>
+      </c>
+      <c r="K108" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="L108" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="M108" t="inlineStr">
+        <is>
+          <t>HYPOTHESIS</t>
+        </is>
+      </c>
+      <c r="Q108" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="R108" t="inlineStr">
+        <is>
+          <t>2026-09-10 · seed · T1</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>LR-08</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>GOM-E un-hedge ∧ kho ≥50%/5d ∧ px −30% → lead [8-9]d</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D109" t="n">
+        <v>1</v>
+      </c>
+      <c r="E109" t="n">
+        <v>0</v>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>AKE:2026-09-10:92fa9c56</t>
+        </is>
+      </c>
+      <c r="K109" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L109" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="M109" t="inlineStr">
+        <is>
+          <t>HYPOTHESIS</t>
+        </is>
+      </c>
+      <c r="Q109" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="R109" t="inlineStr">
+        <is>
+          <t>2026-09-10 · seed · T1</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>LR-09</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>G3(b) vế "OI-build" sai; seat-lift = pos_ramp trên OI phẳng; div TĂNG từ ≤0.5</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>B/C</t>
+        </is>
+      </c>
+      <c r="D110" t="n">
+        <v>3</v>
+      </c>
+      <c r="E110" t="n">
+        <v>0</v>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>AKE:2026-09-10:92fa9c56, CYS:2026-09-10:af073e64, PROM:2026-09-10:b50b1f68</t>
+        </is>
+      </c>
+      <c r="K110" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L110" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="M110" t="inlineStr">
+        <is>
+          <t>CANDIDATE</t>
+        </is>
+      </c>
+      <c r="Q110" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="R110" t="inlineStr">
+        <is>
+          <t>2026-09-10 · seed · T1 (→ AMD-05 B3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>LR-10</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>acc_r sập ≥[40-50%]/≤3d quanh ignition = xác nhận muộn (không phân biệt E)</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="D111" t="n">
+        <v>13</v>
+      </c>
+      <c r="E111" t="n">
+        <v>0</v>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>AKE:2026-09-10:92fa9c56, TUT:2026-09-10:4ab482bc, BANK:2026-09-10:7e520f40, BTW:2026-09-10:ffe6b6de, BTR:2026-09-10:c988194e, CAP:2026-09-10:2695bc3f, ON:2026-09-10:4e0e3a7a, HEMI:2026-09-10:4238441f, BULLA:2026-09-10:deb0b268, 龙虾:2026-09-10:2b727853, UAI:2026-09-10:af767473, CYS:2026-09-10:af073e64, PROM:2026-09-10:b50b1f68</t>
+        </is>
+      </c>
+      <c r="K111" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L111" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="M111" t="inlineStr">
+        <is>
+          <t>RULE-XÁC-NHẬN</t>
+        </is>
+      </c>
+      <c r="N111" t="inlineStr">
+        <is>
+          <t>descriptive:40-50</t>
+        </is>
+      </c>
+      <c r="O111" t="inlineStr">
+        <is>
+          <t>Tiên</t>
+        </is>
+      </c>
+      <c r="P111" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="Q111" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="R111" t="inlineStr">
+        <is>
+          <t>2026-09-10 · seed · T1 · Tiên ký 10/09</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>LR-11</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>decay/S5 SUPPRESSED cần TTL hoặc vế đảo (OI +[40%]/14d trên giá phẳng)</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>C/D</t>
+        </is>
+      </c>
+      <c r="D112" t="n">
+        <v>1</v>
+      </c>
+      <c r="E112" t="n">
+        <v>0</v>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>BTW:2026-09-10:ffe6b6de</t>
+        </is>
+      </c>
+      <c r="K112" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L112" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="M112" t="inlineStr">
+        <is>
+          <t>HYPOTHESIS</t>
+        </is>
+      </c>
+      <c r="Q112" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="R112" t="inlineStr">
+        <is>
+          <t>2026-09-10 · seed · T1</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>LR-12</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>kho RÚT trước pump ở loài A; kho NẠP ở loài B/C/D — đọc theo loài</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>A vs B/C/D</t>
+        </is>
+      </c>
+      <c r="D113" t="n">
+        <v>6</v>
+      </c>
+      <c r="E113" t="n">
+        <v>0</v>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>CYS:2026-09-10:af073e64, 龙虾:2026-09-10:2b727853, UAI:2026-09-10:af767473, AKE:2026-09-10:92fa9c56, HEMI:2026-09-10:4238441f, BTR:2026-09-10:c988194e</t>
+        </is>
+      </c>
+      <c r="J113" t="inlineStr">
+        <is>
+          <t>BANK:2026-09-10:[CHART-READ], PROM:2026-09-10:[CHART-READ], CAP:2026-09-10:[CHART-READ], ON:2026-09-10:[CHART-READ]</t>
+        </is>
+      </c>
+      <c r="K113" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L113" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="M113" t="inlineStr">
+        <is>
+          <t>CANDIDATE</t>
+        </is>
+      </c>
+      <c r="Q113" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="R113" t="inlineStr">
+        <is>
+          <t>2026-09-10 · seed · T1 · 4 ảnh CHART-READ trong cases_pending (BANK/PROM/CAP/ON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>LR-13</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>unhedge-event = div_avg3 vượt 0.5→[0.7] ≤3d ∧ Δacc ≤−[15%] ∧ |Δpos| ≤[10%] (crowd rời); Δpos ≥+[20%] = whale đổi ghế (bẫy)</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D114" t="n">
+        <v>3</v>
+      </c>
+      <c r="E114" t="n">
+        <v>0</v>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>BTR:2026-09-10:c988194e, BULLA:2026-09-10:deb0b268, UAI:2026-09-10:af767473</t>
+        </is>
+      </c>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>SOPH:2026-06-27:344cf3c8, SOPH:2026-07-12:344cf3c8, SOPH:2026-08-08:344cf3c8</t>
+        </is>
+      </c>
+      <c r="K114" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="L114" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="M114" t="inlineStr">
+        <is>
+          <t>CANDIDATE</t>
+        </is>
+      </c>
+      <c r="Q114" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="R114" t="inlineStr">
+        <is>
+          <t>2026-09-10 · seed · T1 · counter 3→0 SOPH×3→TN</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>LR-14</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>deposit-in-pump không kết thúc sóng nếu pos_r hồi ≥ trước-flush ≤3d</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="D115" t="n">
+        <v>1</v>
+      </c>
+      <c r="E115" t="n">
+        <v>0</v>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>HEMI:2026-09-10:4238441f</t>
+        </is>
+      </c>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>BANK:2026-09-10:7e520f40, BTR:2026-09-10:c988194e, ON:2026-09-10:4e0e3a7a, 龙虾:2026-09-10:2b727853</t>
+        </is>
+      </c>
+      <c r="K115" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L115" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="M115" t="inlineStr">
+        <is>
+          <t>HYPOTHESIS</t>
+        </is>
+      </c>
+      <c r="Q115" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="R115" t="inlineStr">
+        <is>
+          <t>2026-09-10 · seed · T1 · counter 4→0 BANK/BTR/ON/龙虾→TN</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>LR-15</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>nến ≥+[35%] ∧ spot/perp ≤[1.2%] ∧ không nến ≥+[10%] trong ≤3d ∧ crowd đảo long D+2-3 = rụng</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="D116" t="n">
+        <v>2</v>
+      </c>
+      <c r="E116" t="n">
+        <v>1</v>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>APR:2026-09-10:2f0918b6, SOPH:2026-09-10:344cf3c8</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>HEMI:2026-09-10:4238441f</t>
+        </is>
+      </c>
+      <c r="K116" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="L116" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="M116" t="inlineStr">
+        <is>
+          <t>HYPOTHESIS</t>
+        </is>
+      </c>
+      <c r="Q116" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="R116" t="inlineStr">
+        <is>
+          <t>2026-09-10 · seed · T1 (R7 in 3 vế, không verdict) · 2026-09-11 · CANDIDATE→HYPOTHESIS · support_n=2&lt;3</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>LR-16</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>GOM-A A1 bắn sau khi crowd bị rửa (div nở do acc sập), không phải khi whale gom</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D117" t="n">
+        <v>3</v>
+      </c>
+      <c r="E117" t="n">
+        <v>0</v>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>HEMI:2026-09-10:4238441f, BULLA:2026-09-10:deb0b268, UAI:2026-09-10:af767473</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>PROM:2026-09-10:b50b1f68</t>
+        </is>
+      </c>
+      <c r="K117" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L117" t="inlineStr">
+        <is>
+          <t>E1</t>
+        </is>
+      </c>
+      <c r="M117" t="inlineStr">
+        <is>
+          <t>CANDIDATE</t>
+        </is>
+      </c>
+      <c r="Q117" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="R117" t="inlineStr">
+        <is>
+          <t>2026-09-10 · seed · T1 · counter 1→0 PROM→NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>LR-17</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>OI trước ignition: giảm ở loài A (CYS −40%, PROM −25%, UAI −27%); build ở loài D (BTW +54%, 龙虾 +64%); phẳng còn lại — OI không phải luật chung</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>A vs D</t>
+        </is>
+      </c>
+      <c r="D118" t="n">
+        <v>5</v>
+      </c>
+      <c r="E118" t="n">
+        <v>0</v>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>CYS:2026-09-10:af073e64, PROM:2026-09-10:b50b1f68, UAI:2026-09-10:af767473, BTW:2026-09-10:ffe6b6de, 龙虾:2026-09-10:2b727853</t>
+        </is>
+      </c>
+      <c r="K118" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L118" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="M118" t="inlineStr">
+        <is>
+          <t>CANDIDATE</t>
+        </is>
+      </c>
+      <c r="Q118" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="R118" t="inlineStr">
+        <is>
+          <t>2026-09-10 · seed · T1</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>LR-18</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>Nansen bal_date trễ [1-3]d: lead từ kho phải trừ; replay không thay findings khi coverage mù</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="D119" t="n">
+        <v>5</v>
+      </c>
+      <c r="E119" t="n">
+        <v>0</v>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>AKE:2026-09-10:92fa9c56, HEMI:2026-09-10:4238441f, BANK:2026-09-10:7e520f40, ON:2026-09-10:4e0e3a7a, APR:2026-09-10:2f0918b6</t>
+        </is>
+      </c>
+      <c r="K119" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L119" t="inlineStr">
+        <is>
+          <t>E1</t>
+        </is>
+      </c>
+      <c r="M119" t="inlineStr">
+        <is>
+          <t>CANDIDATE</t>
+        </is>
+      </c>
+      <c r="Q119" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="R119" t="inlineStr">
+        <is>
+          <t>2026-09-10 · seed · T1 (operator explicit: CANDIDATE, không RULE)</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>LR-20</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>hedge-struct ≥[30]d không unhedge-event = CHRONIC (FP); List-A cần TTL</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D120" t="n">
+        <v>1</v>
+      </c>
+      <c r="E120" t="n">
+        <v>0</v>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>SOPH:2026-09-10:344cf3c8</t>
+        </is>
+      </c>
+      <c r="K120" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="L120" t="inlineStr">
+        <is>
+          <t>E1</t>
+        </is>
+      </c>
+      <c r="M120" t="inlineStr">
+        <is>
+          <t>HYPOTHESIS</t>
+        </is>
+      </c>
+      <c r="Q120" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="R120" t="inlineStr">
+        <is>
+          <t>2026-09-10 · seed · T1 (→ A3/B4) · 2026-09-11 · CANDIDATE→HYPOTHESIS · support_n=1&lt;3</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>L-28 am.1</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>whales_config căn cước bằng giá contract</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>MIGRATION-CLASSIFIER-28-09</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>nguồn ngoài neo căn cước = khớp giá CỦA ĐỊA CHỈ với perp (≤[5×]); giá theo symbol (spot/Alpha-symbol) là sanity-circle, không dùng cho căn cước/DEAD; symbol, Alpha entry, CoinGecko chỉ là ứng viên. Ca: ARX · STAR · BOB · ONE (trùng contract với CROSS) · PLAY · TAC.</t>
         </is>
       </c>
     </row>
@@ -5640,4 +6732,1377 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K28"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>token</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>display_token</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>path</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>case_xlsx_md5_after</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>addendum_count</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>ledger_count</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>loài</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>trạng_thái</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>added_at_utc</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>kr_share_14d_pct</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>kr_led</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>BANK</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>BANK</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>docs/case_files/BANK/</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>b550820d70cc0eb46b3d1defea398409</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>proven·hedge</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>proven</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>2026-09-10T10:11:07.862843+00:00</t>
+        </is>
+      </c>
+      <c r="J2" t="n">
+        <v>39.2</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>TUT</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>TUT</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>docs/case_files/TUT/</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>8580030a491520526b70937c401934ec</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>proven</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>proven</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>2026-09-10T10:11:07.862843+00:00</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>N/A-NOT-IN-KR-SWEEP</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>AKE</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>AKE</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>docs/case_files/AKE/</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>8b86051c70009442c354238bebca8e8b</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>proven·hedge</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>proven</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>2026-09-10T10:11:07.862843+00:00</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>N/A-NOT-IN-KR-SWEEP</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>BTW</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>BTW</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>docs/case_files/BTW/</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>be21051483eaa5b01875d82844ef6b09</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>proven</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>proven</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>2026-09-10T10:11:07.862843+00:00</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>N/A-NOT-IN-KR-SWEEP</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>CYS</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>CYS</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>docs/case_files/CYS/</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>5603f3dbcfc598cc4865e3ff5991c8bc</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" t="n">
+        <v>2</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>proven</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>proven</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>2026-09-10T10:11:07.862843+00:00</t>
+        </is>
+      </c>
+      <c r="J6" t="n">
+        <v>73.29000000000001</v>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>KR-DẪN</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>BTR</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>BTR</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>docs/case_files/BTR/</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>7dc7191c1854e7c5649e92af1ee13fdb</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>đối chứng</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>đối chứng</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>2026-09-10T10:11:07.862843+00:00</t>
+        </is>
+      </c>
+      <c r="J7" t="n">
+        <v>83.3</v>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>KR-DẪN</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>CAP</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>CAP</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>docs/case_files/CAP/</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>c5ecf59044d31002f77e825adaf58300</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>2026-09-10T10:11:07.862843+00:00</t>
+        </is>
+      </c>
+      <c r="J8" t="n">
+        <v>55.67</v>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>KR-DẪN</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>docs/case_files/ON/</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>c550d14ab2e282e096fee1bc66d9cfb2</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>proven·hedge</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>proven</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>2026-09-10T10:11:07.862843+00:00</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>N/A-NOT-IN-KR-SWEEP</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>APR</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>APR</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>docs/case_files/APR/</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>0750f1df6c735590825e632e22bc03ec</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" t="n">
+        <v>1</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>đối chứng·1-cột</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>đối chứng</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>2026-09-10T10:11:07.862843+00:00</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>N/A-NOT-IN-KR-SWEEP</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>HEMI</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>HEMI</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>docs/case_files/HEMI/</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>ff0e2eb5e004b48b02e1973fe3f31bb7</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" t="n">
+        <v>1</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>proven·hedge</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>proven</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>2026-09-10T10:11:07.862843+00:00</t>
+        </is>
+      </c>
+      <c r="J11" t="n">
+        <v>37.14</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>BULLA</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>BULLA</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>docs/case_files/BULLA/</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>c0b0f50746d16504327ef986110eca86</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" t="n">
+        <v>1</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>proven·sống·2-sóng</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>sống (sóng-2 mở)</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>2026-09-10T10:11:07.862843+00:00</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>N/A-NOT-IN-KR-SWEEP</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>PROM</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>PROM</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>docs/case_files/PROM/</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>820fe247aae802cdabefb83f1687150e</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" t="n">
+        <v>1</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>đối chứng</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>đối chứng</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>2026-09-10T10:11:07.862843+00:00</t>
+        </is>
+      </c>
+      <c r="J13" t="n">
+        <v>31.95</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>LOBSTER</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>龙虾</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>docs/case_files/LOBSTER/</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>1566884da03567be5d78e9783dd6c49a</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>1</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>proven·kho90%</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>proven</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>2026-09-10T10:11:07.862843+00:00</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>N/A-NOT-IN-KR-SWEEP</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>UAI</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>UAI</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>docs/case_files/UAI/</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>4fa8599e6fa2c238d275ef5cc701861a</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>1</v>
+      </c>
+      <c r="F15" t="n">
+        <v>1</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>proven·hedge</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>proven</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>2026-09-10T10:11:07.862843+00:00</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>N/A-NOT-IN-KR-SWEEP</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>SOPH</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>SOPH</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>docs/case_files/SOPH/</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>cf7c8c78b9eff091993a2a635f13e048</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F16" t="n">
+        <v>1</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>đối chứng·1-cột</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>đối chứng</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>2026-09-10T10:11:07.862843+00:00</t>
+        </is>
+      </c>
+      <c r="J16" t="n">
+        <v>83.19</v>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>KR-DẪN</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>LIGHT</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>LIGHT</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>docs/case_files/LIGHT/</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>4bfcca85346edb0822fd36291af19501</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>1</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>SỐNG [KHUÔN-draft] · GRIND-DEPOSIT</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>SỐNG</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>2026-09-11T08:05:46Z</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>N/A-NOT-IN-KR-SWEEP</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>BROCCOLIF3B</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>BROCCOLIF3B</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>docs/case_files/BROCCOLIF3B/</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>82dd9b10244f0f9356811786267899ec</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>SỐNG [KHUÔN-draft] · meme 1Y · Nansen NOT-TRACKED</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>SỐNG</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>2026-09-11T08:33:44Z</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>N/A-NOT-IN-KR-SWEEP</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>docs/case_files/AT/</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>7e2b5e3553942bd1910001e6eb563cc4</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>1</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>SỐNG [KHUÔN-draft] · 2M window</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>SỐNG</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>2026-09-11T08:48:48Z</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>N/A-NOT-IN-KR-SWEEP</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>BASED</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>BASED</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>docs/case_files/BASED/</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>9be1966928a0d415f97d7b40acc7b673</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>1</v>
+      </c>
+      <c r="F20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>SỐNG [KHUÔN-draft] · census H1 26/07 MED</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>SỐNG</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>2026-09-11T09:05:55Z</t>
+        </is>
+      </c>
+      <c r="J20" t="n">
+        <v>49.12</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>MARSCOIN</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>MARSCOIN</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>docs/case_files/MARSCOIN/</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>eb47a65c80958f776d7976fd82b7670c</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>1</v>
+      </c>
+      <c r="F21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>SỐNG [KHUÔN-draft] · perp 9d · Nansen NOT-TRACKED · meme 100%</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>SỐNG</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>2026-09-11T09:30:27Z</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>N/A-NOT-IN-KR-SWEEP</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>HYPER</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>HYPER</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>docs/case_files/HYPER/</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>755ee510a52db522bf2d03b30ead913e</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>1</v>
+      </c>
+      <c r="F22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>SỐNG [KHUÔN-draft] · Hyperlane BSC · Alpha delisted · kho TRACKED</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>SỐNG</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>2026-09-11T14:34:57Z</t>
+        </is>
+      </c>
+      <c r="J22" t="n">
+        <v>38.95</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>RED</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>RED</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>docs/case_files/RED/</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>047c6d1edd02c779080470a53025bfde</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>1</v>
+      </c>
+      <c r="F23" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>SỐNG [KHUÔN-draft] · perp+spot · NO Alpha · Nansen NOT-TRACKED</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>SỐNG</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>2026-09-11T14:50:04Z</t>
+        </is>
+      </c>
+      <c r="J23" t="n">
+        <v>47.9</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>MITO</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>MITO</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>docs/case_files/MITO/</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>e64fb345b398cafcb193eb669204c207</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>1</v>
+      </c>
+      <c r="F24" t="n">
+        <v>0</v>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>SỐNG [KHUÔN-draft] · XẢ-WATCH · D7=3/8 · fork A/B/C</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>SỐNG</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>2026-09-11T22:55:39Z</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>N/A-NOT-IN-KR-SWEEP</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>WTMLL</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>我踏马来了</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>docs/case_files/WTMLL/</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>abd9050a3b01c85bfd654fe45b99569b</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>1</v>
+      </c>
+      <c r="F25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>SỐNG [KHUÔN-draft] · Chinese-family meme · Nansen TRACKED</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>SỐNG</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>2026-09-12T14:20:43Z</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>N/A-NOT-IN-KR-SWEEP</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>ARX</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>ARX</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>docs/case_files/ARX/</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>b6f7d445b8a8bc91a41c8f744a4bdba0</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>1</v>
+      </c>
+      <c r="F26" t="n">
+        <v>0</v>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>SỐNG [KHUÔN-draft] · Arcium · Nansen NOT-TRACKED · spot N/A</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>SỐNG</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>2026-09-12T15:02:44Z</t>
+        </is>
+      </c>
+      <c r="J26" t="n">
+        <v>72.54000000000001</v>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>KR-DẪN</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>POWER</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>POWER</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>docs/case_files/POWER/</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>63ef70aa024d796b65dc621d4c570ce7</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>1</v>
+      </c>
+      <c r="F27" t="n">
+        <v>0</v>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>SỐNG [KHUÔN-draft] · Power Protocol · cover-event 02/09</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>SỐNG</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>2026-09-13T08:04:30Z</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>N/A-NOT-IN-KR-SWEEP</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>LSK</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>LSK</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>docs/case_files/LSK/</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>8a65c3e6798db9fdcdc0fa70eb712b1b</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>1</v>
+      </c>
+      <c r="F28" t="n">
+        <v>0</v>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>SỐNG [KHUÔN-draft] · Lisk L1/L2 · spot TRADING · B-top 08-13→08-17</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>SỐNG</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>2026-09-13T12:12:27Z</t>
+        </is>
+      </c>
+      <c r="J28" t="n">
+        <v>71.54000000000001</v>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>KR-DẪN</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
L-81/L-82 promoted from LR-05/LR-10 · ký chat Tiến 28/09
L-81 (row 122): taker_buy pin xuyên markup · descriptive:55 · from LR-05
L-82 (row 123): acc_r sập quanh ignition · descriptive:40-50 · from LR-10
LR-05 (row 106) · LR-10 (row 111): status → PROMOTED→L-8x + changelog append

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/case_files/CASE_INDEX.xlsx
+++ b/docs/case_files/CASE_INDEX.xlsx
@@ -1742,7 +1742,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R121"/>
+  <dimension ref="A1:R123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -5552,7 +5552,7 @@
       </c>
       <c r="M106" t="inlineStr">
         <is>
-          <t>RULE-XÁC-NHẬN</t>
+          <t>PROMOTED→L-81</t>
         </is>
       </c>
       <c r="N106" t="inlineStr">
@@ -5577,7 +5577,7 @@
       </c>
       <c r="R106" t="inlineStr">
         <is>
-          <t>2026-09-10 · seed · T1 · Tiên ký 10/09</t>
+          <t>2026-09-10 · seed · T1 · Tiên ký 10/09 · 2026-09-28 promoted</t>
         </is>
       </c>
     </row>
@@ -5842,7 +5842,7 @@
       </c>
       <c r="M111" t="inlineStr">
         <is>
-          <t>RULE-XÁC-NHẬN</t>
+          <t>PROMOTED→L-82</t>
         </is>
       </c>
       <c r="N111" t="inlineStr">
@@ -5867,7 +5867,7 @@
       </c>
       <c r="R111" t="inlineStr">
         <is>
-          <t>2026-09-10 · seed · T1 · Tiên ký 10/09</t>
+          <t>2026-09-10 · seed · T1 · Tiên ký 10/09 · 2026-09-28 promoted</t>
         </is>
       </c>
     </row>
@@ -6392,6 +6392,50 @@
       <c r="D121" t="inlineStr">
         <is>
           <t>nguồn ngoài neo căn cước = khớp giá CỦA ĐỊA CHỈ với perp (≤[5×]); giá theo symbol (spot/Alpha-symbol) là sanity-circle, không dùng cho căn cước/DEAD; symbol, Alpha entry, CoinGecko chỉ là ứng viên. Ca: ARX · STAR · BOB · ONE (trùng contract với CROSS) · PLAY · TAC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>L-81</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>taker_buy pin xuyên markup</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>PROMOTE-LR-05-28-09</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>taker_buy &lt;[55%] xuyên markup (≤1 ngày eve) · ngưỡng descriptive:55 · evidence_class=E2 · support_n=13 · counter_n=0 · gate_binding=N · promoted from LR-05 (gieo 10/09 · bada4e50) · ký chat Tiến 28/09</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>L-82</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>acc_r sập quanh ignition = xác nhận muộn</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>PROMOTE-LR-10-28-09</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>acc_r sập ≥[40-50%]/≤3d quanh ignition = xác nhận muộn (không phân biệt E) · ngưỡng descriptive:40-50 · evidence_class=E2 · support_n=13 · counter_n=0 · gate_binding=N · promoted from LR-10 (gieo 10/09 · bada4e50) · ký chat Tiến 28/09</t>
         </is>
       </c>
     </row>

</xml_diff>